<commit_message>
working on one Data cruncher L3 to rule them all
generally works, but some data is missing from L3 step 31
</commit_message>
<xml_diff>
--- a/scratch/FormattedCutTableL3_template_md.xlsx
+++ b/scratch/FormattedCutTableL3_template_md.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/sam mac stove data/DOE Data/lab tests/5 stoves comparison/all stoves/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8BD6D45-0461-FB40-A2CE-B5D9D9538A35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78495D29-2A09-8048-9AA7-37F3223F0FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1060" yWindow="540" windowWidth="27220" windowHeight="20260" xr2:uid="{1837E1AF-DB18-D64C-9443-79C0B4F568AD}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2951" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2946" uniqueCount="270">
   <si>
     <t>Metrics</t>
   </si>
@@ -587,9 +587,6 @@
   </si>
   <si>
     <t>Control temperature</t>
-  </si>
-  <si>
-    <t>C</t>
   </si>
   <si>
     <t>STC2_L1</t>
@@ -1260,7 +1257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1336,11 +1333,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1669,7 +1661,7 @@
     <col min="11" max="11" width="11.83203125" style="56" customWidth="1"/>
     <col min="12" max="17" width="11.83203125" style="1" customWidth="1"/>
     <col min="18" max="18" width="8.83203125" style="2" customWidth="1"/>
-    <col min="19" max="23" width="8.83203125" style="60" customWidth="1"/>
+    <col min="19" max="23" width="8.83203125" style="1" customWidth="1"/>
     <col min="24" max="24" width="9.6640625" style="1" customWidth="1"/>
     <col min="25" max="25" width="7" style="1" customWidth="1"/>
     <col min="26" max="26" width="8.33203125" style="1" customWidth="1"/>
@@ -1722,7 +1714,7 @@
       <c r="AH1" s="17"/>
       <c r="AI1" s="17"/>
       <c r="AJ1" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AP1" s="17" t="s">
         <v>171</v>
@@ -1835,7 +1827,7 @@
         <v>153</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J3" s="16" t="s">
         <v>142</v>
@@ -1859,7 +1851,7 @@
         <v>157</v>
       </c>
       <c r="Q3" s="15" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="R3" t="s">
         <v>144</v>
@@ -1877,115 +1869,115 @@
         <v>163</v>
       </c>
       <c r="W3" s="15" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="X3" t="s">
         <v>145</v>
       </c>
       <c r="Y3" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z3" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="Z3" s="15" t="s">
+      <c r="AA3" s="15" t="s">
         <v>220</v>
       </c>
-      <c r="AA3" s="15" t="s">
+      <c r="AB3" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="AB3" s="15" t="s">
-        <v>222</v>
-      </c>
-      <c r="AC3" s="62" t="s">
-        <v>246</v>
+      <c r="AC3" t="s">
+        <v>245</v>
       </c>
       <c r="AD3" t="s">
         <v>146</v>
       </c>
       <c r="AE3" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="AF3" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="AF3" s="15" t="s">
+      <c r="AG3" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="AG3" s="15" t="s">
+      <c r="AH3" s="15" t="s">
         <v>225</v>
       </c>
-      <c r="AH3" s="15" t="s">
+      <c r="AI3" t="s">
+        <v>246</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>201</v>
+      </c>
+      <c r="AK3" s="15" t="s">
         <v>226</v>
       </c>
-      <c r="AI3" s="62" t="s">
+      <c r="AL3" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="AM3" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="AN3" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="AO3" t="s">
         <v>247</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>202</v>
-      </c>
-      <c r="AK3" s="15" t="s">
-        <v>227</v>
-      </c>
-      <c r="AL3" s="15" t="s">
-        <v>228</v>
-      </c>
-      <c r="AM3" s="15" t="s">
-        <v>229</v>
-      </c>
-      <c r="AN3" s="15" t="s">
-        <v>230</v>
-      </c>
-      <c r="AO3" s="62" t="s">
-        <v>248</v>
       </c>
       <c r="AP3" t="s">
         <v>147</v>
       </c>
       <c r="AQ3" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="AR3" s="15" t="s">
         <v>231</v>
       </c>
-      <c r="AR3" s="15" t="s">
+      <c r="AS3" s="15" t="s">
         <v>232</v>
       </c>
-      <c r="AS3" s="15" t="s">
+      <c r="AT3" s="15" t="s">
         <v>233</v>
       </c>
-      <c r="AT3" s="15" t="s">
-        <v>234</v>
-      </c>
-      <c r="AU3" s="62" t="s">
-        <v>249</v>
+      <c r="AU3" t="s">
+        <v>248</v>
       </c>
       <c r="AV3" t="s">
         <v>164</v>
       </c>
       <c r="AW3" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="AX3" s="15" t="s">
         <v>235</v>
       </c>
-      <c r="AX3" s="15" t="s">
+      <c r="AY3" s="15" t="s">
         <v>236</v>
       </c>
-      <c r="AY3" s="15" t="s">
+      <c r="AZ3" s="15" t="s">
         <v>237</v>
       </c>
-      <c r="AZ3" s="15" t="s">
-        <v>238</v>
-      </c>
-      <c r="BA3" s="62" t="s">
-        <v>250</v>
+      <c r="BA3" t="s">
+        <v>249</v>
       </c>
       <c r="BB3" t="s">
         <v>148</v>
       </c>
       <c r="BC3" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="BD3" s="15" t="s">
         <v>239</v>
       </c>
-      <c r="BD3" s="15" t="s">
+      <c r="BE3" s="15" t="s">
         <v>240</v>
       </c>
-      <c r="BE3" s="15" t="s">
+      <c r="BF3" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="BF3" s="15" t="s">
-        <v>242</v>
-      </c>
       <c r="BG3" s="13" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="BH3" t="s">
         <v>149</v>
@@ -4613,7 +4605,7 @@
       <c r="F33" s="29"/>
       <c r="G33" s="29"/>
       <c r="H33" s="29"/>
-      <c r="I33" s="59"/>
+      <c r="I33"/>
       <c r="J33" s="18"/>
       <c r="K33" s="32"/>
       <c r="L33" s="26"/>
@@ -4621,42 +4613,42 @@
       <c r="N33" s="29"/>
       <c r="O33" s="29"/>
       <c r="P33" s="29"/>
-      <c r="Q33" s="59"/>
+      <c r="Q33"/>
       <c r="S33" s="52"/>
       <c r="T33" s="29"/>
       <c r="U33" s="29"/>
       <c r="V33" s="29"/>
-      <c r="W33" s="59"/>
+      <c r="W33"/>
       <c r="Y33" s="52"/>
       <c r="Z33" s="29"/>
       <c r="AA33" s="29"/>
       <c r="AB33" s="29"/>
-      <c r="AC33" s="59"/>
+      <c r="AC33"/>
       <c r="AE33" s="52"/>
       <c r="AF33" s="29"/>
       <c r="AG33" s="29"/>
       <c r="AH33" s="29"/>
-      <c r="AI33" s="59"/>
+      <c r="AI33"/>
       <c r="AK33" s="52"/>
       <c r="AL33" s="29"/>
       <c r="AM33" s="29"/>
       <c r="AN33" s="29"/>
-      <c r="AO33" s="59"/>
+      <c r="AO33"/>
       <c r="AQ33" s="52"/>
       <c r="AR33" s="29"/>
       <c r="AS33" s="29"/>
       <c r="AT33" s="29"/>
-      <c r="AU33" s="59"/>
+      <c r="AU33"/>
       <c r="AW33" s="52"/>
       <c r="AX33" s="29"/>
       <c r="AY33" s="29"/>
       <c r="AZ33" s="29"/>
-      <c r="BA33" s="59"/>
+      <c r="BA33"/>
       <c r="BC33" s="52"/>
       <c r="BD33" s="29"/>
       <c r="BE33" s="29"/>
       <c r="BF33" s="29"/>
-      <c r="BG33" s="59"/>
+      <c r="BG33"/>
     </row>
     <row r="34" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C34" s="17"/>
@@ -5757,7 +5749,7 @@
     </row>
     <row r="46" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C46" s="27" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D46" s="25"/>
       <c r="E46" s="51"/>
@@ -5995,10 +5987,10 @@
         <v>132</v>
       </c>
       <c r="H50" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J50" s="38"/>
       <c r="K50" s="39" t="str">
@@ -6016,10 +6008,10 @@
         <v>132</v>
       </c>
       <c r="P50" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="Q50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="S50" s="51" t="s">
         <v>26</v>
@@ -6031,10 +6023,10 @@
         <v>132</v>
       </c>
       <c r="V50" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="W50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Y50" s="51" t="s">
         <v>26</v>
@@ -6046,10 +6038,10 @@
         <v>132</v>
       </c>
       <c r="AB50" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AC50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AE50" s="51" t="s">
         <v>26</v>
@@ -6061,10 +6053,10 @@
         <v>132</v>
       </c>
       <c r="AH50" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AI50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AK50" s="51" t="s">
         <v>26</v>
@@ -6076,10 +6068,10 @@
         <v>132</v>
       </c>
       <c r="AN50" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AO50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AQ50" s="51" t="s">
         <v>26</v>
@@ -6091,10 +6083,10 @@
         <v>132</v>
       </c>
       <c r="AT50" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AU50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AW50" s="51" t="s">
         <v>26</v>
@@ -6106,10 +6098,10 @@
         <v>132</v>
       </c>
       <c r="AZ50" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="BA50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="BC50" s="51" t="s">
         <v>26</v>
@@ -6121,10 +6113,10 @@
         <v>132</v>
       </c>
       <c r="BF50" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="BG50" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="51" spans="3:59" s="6" customFormat="1" x14ac:dyDescent="0.2">
@@ -7911,42 +7903,42 @@
       <c r="N69" s="29"/>
       <c r="O69" s="29"/>
       <c r="P69" s="29"/>
-      <c r="Q69" s="59"/>
+      <c r="Q69"/>
       <c r="S69" s="52"/>
       <c r="T69" s="29"/>
       <c r="U69" s="29"/>
       <c r="V69" s="29"/>
-      <c r="W69" s="59"/>
+      <c r="W69"/>
       <c r="Y69" s="52"/>
       <c r="Z69" s="29"/>
       <c r="AA69" s="29"/>
       <c r="AB69" s="29"/>
-      <c r="AC69" s="59"/>
+      <c r="AC69"/>
       <c r="AE69" s="52"/>
       <c r="AF69" s="29"/>
       <c r="AG69" s="29"/>
       <c r="AH69" s="29"/>
-      <c r="AI69" s="59"/>
+      <c r="AI69"/>
       <c r="AK69" s="52"/>
       <c r="AL69" s="29"/>
       <c r="AM69" s="29"/>
       <c r="AN69" s="29"/>
-      <c r="AO69" s="59"/>
+      <c r="AO69"/>
       <c r="AQ69" s="52"/>
       <c r="AR69" s="29"/>
       <c r="AS69" s="29"/>
       <c r="AT69" s="29"/>
-      <c r="AU69" s="59"/>
+      <c r="AU69"/>
       <c r="AW69" s="52"/>
       <c r="AX69" s="29"/>
       <c r="AY69" s="29"/>
       <c r="AZ69" s="29"/>
-      <c r="BA69" s="59"/>
+      <c r="BA69"/>
       <c r="BC69" s="52"/>
       <c r="BD69" s="29"/>
       <c r="BE69" s="29"/>
       <c r="BF69" s="29"/>
-      <c r="BG69" s="59"/>
+      <c r="BG69"/>
     </row>
     <row r="70" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C70" s="17"/>
@@ -9767,42 +9759,42 @@
       <c r="N86" s="29"/>
       <c r="O86" s="29"/>
       <c r="P86" s="43"/>
-      <c r="Q86" s="61"/>
+      <c r="Q86" s="13"/>
       <c r="S86" s="52"/>
       <c r="T86" s="29"/>
       <c r="U86" s="29"/>
       <c r="V86" s="43"/>
-      <c r="W86" s="61"/>
+      <c r="W86" s="13"/>
       <c r="Y86" s="52"/>
       <c r="Z86" s="29"/>
       <c r="AA86" s="29"/>
       <c r="AB86" s="43"/>
-      <c r="AC86" s="61"/>
+      <c r="AC86" s="13"/>
       <c r="AE86" s="52"/>
       <c r="AF86" s="29"/>
       <c r="AG86" s="29"/>
       <c r="AH86" s="43"/>
-      <c r="AI86" s="61"/>
+      <c r="AI86" s="13"/>
       <c r="AK86" s="52"/>
       <c r="AL86" s="29"/>
       <c r="AM86" s="29"/>
       <c r="AN86" s="43"/>
-      <c r="AO86" s="61"/>
+      <c r="AO86" s="13"/>
       <c r="AQ86" s="52"/>
       <c r="AR86" s="29"/>
       <c r="AS86" s="29"/>
       <c r="AT86" s="43"/>
-      <c r="AU86" s="61"/>
+      <c r="AU86" s="13"/>
       <c r="AW86" s="52"/>
       <c r="AX86" s="29"/>
       <c r="AY86" s="29"/>
       <c r="AZ86" s="43"/>
-      <c r="BA86" s="61"/>
+      <c r="BA86" s="13"/>
       <c r="BC86" s="52"/>
       <c r="BD86" s="29"/>
       <c r="BE86" s="29"/>
       <c r="BF86" s="43"/>
-      <c r="BG86" s="61"/>
+      <c r="BG86" s="13"/>
     </row>
     <row r="87" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C87" s="17"/>
@@ -10662,10 +10654,10 @@
       <c r="F96"/>
       <c r="G96"/>
       <c r="H96" t="s">
+        <v>254</v>
+      </c>
+      <c r="I96" t="s">
         <v>255</v>
-      </c>
-      <c r="I96" t="s">
-        <v>256</v>
       </c>
       <c r="J96" s="18"/>
       <c r="K96" s="32"/>
@@ -10676,10 +10668,10 @@
       <c r="N96"/>
       <c r="O96"/>
       <c r="P96" t="s">
+        <v>254</v>
+      </c>
+      <c r="Q96" t="s">
         <v>255</v>
-      </c>
-      <c r="Q96" t="s">
-        <v>256</v>
       </c>
       <c r="S96" s="51" t="s">
         <v>124</v>
@@ -10687,10 +10679,10 @@
       <c r="T96"/>
       <c r="U96"/>
       <c r="V96" t="s">
+        <v>254</v>
+      </c>
+      <c r="W96" t="s">
         <v>255</v>
-      </c>
-      <c r="W96" t="s">
-        <v>256</v>
       </c>
       <c r="Y96" s="51" t="s">
         <v>124</v>
@@ -10698,10 +10690,10 @@
       <c r="Z96"/>
       <c r="AA96"/>
       <c r="AB96" t="s">
+        <v>254</v>
+      </c>
+      <c r="AC96" t="s">
         <v>255</v>
-      </c>
-      <c r="AC96" t="s">
-        <v>256</v>
       </c>
       <c r="AE96" s="51" t="s">
         <v>124</v>
@@ -10709,10 +10701,10 @@
       <c r="AF96"/>
       <c r="AG96"/>
       <c r="AH96" t="s">
+        <v>254</v>
+      </c>
+      <c r="AI96" t="s">
         <v>255</v>
-      </c>
-      <c r="AI96" t="s">
-        <v>256</v>
       </c>
       <c r="AK96" s="51" t="s">
         <v>124</v>
@@ -10720,10 +10712,10 @@
       <c r="AL96"/>
       <c r="AM96"/>
       <c r="AN96" t="s">
+        <v>254</v>
+      </c>
+      <c r="AO96" t="s">
         <v>255</v>
-      </c>
-      <c r="AO96" t="s">
-        <v>256</v>
       </c>
       <c r="AQ96" s="51" t="s">
         <v>124</v>
@@ -10731,10 +10723,10 @@
       <c r="AR96"/>
       <c r="AS96"/>
       <c r="AT96" t="s">
+        <v>254</v>
+      </c>
+      <c r="AU96" t="s">
         <v>255</v>
-      </c>
-      <c r="AU96" t="s">
-        <v>256</v>
       </c>
       <c r="AW96" s="51" t="s">
         <v>124</v>
@@ -10742,10 +10734,10 @@
       <c r="AX96"/>
       <c r="AY96"/>
       <c r="AZ96" t="s">
+        <v>254</v>
+      </c>
+      <c r="BA96" t="s">
         <v>255</v>
-      </c>
-      <c r="BA96" t="s">
-        <v>256</v>
       </c>
       <c r="BC96" s="51" t="s">
         <v>124</v>
@@ -10753,10 +10745,10 @@
       <c r="BD96"/>
       <c r="BE96"/>
       <c r="BF96" t="s">
+        <v>254</v>
+      </c>
+      <c r="BG96" t="s">
         <v>255</v>
-      </c>
-      <c r="BG96" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="97" spans="3:59" x14ac:dyDescent="0.2">
@@ -12695,10 +12687,10 @@
       <c r="F121"/>
       <c r="G121"/>
       <c r="H121" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I121" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J121" s="18"/>
       <c r="K121" s="32"/>
@@ -12707,73 +12699,73 @@
       <c r="N121"/>
       <c r="O121"/>
       <c r="P121" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="Q121" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="S121" s="51"/>
       <c r="T121"/>
       <c r="U121"/>
       <c r="V121" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="W121" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Y121" s="51"/>
       <c r="Z121"/>
       <c r="AA121"/>
       <c r="AB121" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AC121" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AE121" s="51"/>
       <c r="AF121"/>
       <c r="AG121"/>
       <c r="AH121" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AI121" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AK121" s="51"/>
       <c r="AL121"/>
       <c r="AM121"/>
       <c r="AN121" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AO121" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AQ121" s="51"/>
       <c r="AR121"/>
       <c r="AS121"/>
       <c r="AT121" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="AU121" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AW121" s="51"/>
       <c r="AX121"/>
       <c r="AY121"/>
       <c r="AZ121" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="BA121" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="BC121" s="51"/>
       <c r="BD121"/>
       <c r="BE121"/>
       <c r="BF121" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="BG121" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="122" spans="3:59" x14ac:dyDescent="0.2">
@@ -13260,7 +13252,7 @@
       <c r="P127" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="Q127" s="61"/>
+      <c r="Q127" s="13"/>
       <c r="S127" s="52" t="s">
         <v>139</v>
       </c>
@@ -13273,7 +13265,7 @@
       <c r="V127" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="W127" s="61"/>
+      <c r="W127" s="13"/>
       <c r="Y127" s="52" t="s">
         <v>139</v>
       </c>
@@ -13286,7 +13278,7 @@
       <c r="AB127" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="AC127" s="61"/>
+      <c r="AC127" s="13"/>
       <c r="AE127" s="52" t="s">
         <v>139</v>
       </c>
@@ -13299,7 +13291,7 @@
       <c r="AH127" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="AI127" s="61"/>
+      <c r="AI127" s="13"/>
       <c r="AK127" s="52" t="s">
         <v>139</v>
       </c>
@@ -13312,7 +13304,7 @@
       <c r="AN127" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="AO127" s="61"/>
+      <c r="AO127" s="13"/>
       <c r="AQ127" s="52" t="s">
         <v>139</v>
       </c>
@@ -13325,7 +13317,7 @@
       <c r="AT127" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="AU127" s="61"/>
+      <c r="AU127" s="13"/>
       <c r="AW127" s="52" t="s">
         <v>139</v>
       </c>
@@ -13338,7 +13330,7 @@
       <c r="AZ127" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="BA127" s="61"/>
+      <c r="BA127" s="13"/>
       <c r="BC127" s="52" t="s">
         <v>139</v>
       </c>
@@ -13351,7 +13343,7 @@
       <c r="BF127" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="BG127" s="61"/>
+      <c r="BG127" s="13"/>
     </row>
     <row r="128" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C128" s="9"/>
@@ -13378,7 +13370,6 @@
         <v>71</v>
       </c>
       <c r="Q128" s="13"/>
-      <c r="S128" s="1"/>
       <c r="T128" s="1">
         <v>1</v>
       </c>
@@ -13469,10 +13460,7 @@
       <c r="M130" s="51"/>
       <c r="O130" s="13"/>
       <c r="S130" s="51"/>
-      <c r="T130" s="1"/>
       <c r="U130" s="13"/>
-      <c r="V130" s="1"/>
-      <c r="W130" s="1"/>
       <c r="Y130" s="51"/>
       <c r="AA130" s="13"/>
       <c r="AE130" s="51"/>
@@ -13491,22 +13479,12 @@
       <c r="D131" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="S131" s="1"/>
-      <c r="T131" s="1"/>
-      <c r="U131" s="1"/>
-      <c r="V131" s="1"/>
-      <c r="W131" s="1"/>
     </row>
     <row r="132" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C132" s="9"/>
       <c r="D132" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="S132" s="1"/>
-      <c r="T132" s="1"/>
-      <c r="U132" s="1"/>
-      <c r="V132" s="1"/>
-      <c r="W132" s="1"/>
     </row>
     <row r="133" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C133" s="9"/>
@@ -13523,10 +13501,10 @@
         <v>130</v>
       </c>
       <c r="H133" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I133" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="M133" s="51" t="s">
         <v>139</v>
@@ -13538,10 +13516,10 @@
         <v>130</v>
       </c>
       <c r="P133" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Q133" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="S133" s="51" t="s">
         <v>139</v>
@@ -13553,10 +13531,10 @@
         <v>130</v>
       </c>
       <c r="V133" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="W133" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Y133" s="51" t="s">
         <v>139</v>
@@ -13568,10 +13546,10 @@
         <v>130</v>
       </c>
       <c r="AB133" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AC133" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AE133" s="51" t="s">
         <v>139</v>
@@ -13592,10 +13570,10 @@
         <v>130</v>
       </c>
       <c r="AN133" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AO133" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AQ133" s="51" t="s">
         <v>139</v>
@@ -13607,10 +13585,10 @@
         <v>130</v>
       </c>
       <c r="AT133" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AU133" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AW133" s="51" t="s">
         <v>139</v>
@@ -13622,10 +13600,10 @@
         <v>130</v>
       </c>
       <c r="AZ133" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="BA133" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="BC133" s="51" t="s">
         <v>139</v>
@@ -13637,10 +13615,10 @@
         <v>130</v>
       </c>
       <c r="BF133" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="BG133" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="134" spans="3:59" x14ac:dyDescent="0.2">
@@ -13648,11 +13626,6 @@
       <c r="D134" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="S134" s="1"/>
-      <c r="T134" s="1"/>
-      <c r="U134" s="1"/>
-      <c r="V134" s="1"/>
-      <c r="W134" s="1"/>
     </row>
     <row r="135" spans="3:59" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C135" s="5" t="s">
@@ -13686,7 +13659,6 @@
       <c r="P136" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="S136" s="1"/>
       <c r="T136" s="1">
         <v>1</v>
       </c>
@@ -13696,7 +13668,6 @@
       <c r="V136" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="W136" s="1"/>
       <c r="Z136" s="1">
         <v>1</v>
       </c>
@@ -13775,7 +13746,6 @@
       <c r="P137" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="S137" s="1"/>
       <c r="T137" s="1">
         <v>1</v>
       </c>
@@ -13785,7 +13755,6 @@
       <c r="V137" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="W137" s="1"/>
       <c r="Z137" s="1">
         <v>1</v>
       </c>
@@ -13864,7 +13833,6 @@
       <c r="P138" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="S138" s="1"/>
       <c r="T138" s="1">
         <v>1</v>
       </c>
@@ -13874,7 +13842,6 @@
       <c r="V138" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="W138" s="1"/>
       <c r="Z138" s="1">
         <v>1</v>
       </c>
@@ -13953,7 +13920,6 @@
       <c r="P139" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="S139" s="1"/>
       <c r="T139" s="1">
         <v>1</v>
       </c>
@@ -13963,7 +13929,6 @@
       <c r="V139" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="W139" s="1"/>
       <c r="Z139" s="1">
         <v>1</v>
       </c>
@@ -14044,7 +14009,6 @@
         <v>78</v>
       </c>
       <c r="Q140"/>
-      <c r="S140" s="1"/>
       <c r="T140" s="1">
         <v>1</v>
       </c>
@@ -14142,15 +14106,12 @@
       <c r="P142" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="S142" s="1"/>
-      <c r="T142" s="1"/>
       <c r="U142" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V142" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="W142" s="1"/>
       <c r="AA142" s="1" t="s">
         <v>130</v>
       </c>
@@ -14205,15 +14166,12 @@
       <c r="P143" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="S143" s="1"/>
-      <c r="T143" s="1"/>
       <c r="U143" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V143" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="W143" s="1"/>
       <c r="AA143" s="1" t="s">
         <v>130</v>
       </c>
@@ -14268,15 +14226,12 @@
       <c r="P144" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="S144" s="1"/>
-      <c r="T144" s="1"/>
       <c r="U144" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V144" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="W144" s="1"/>
       <c r="AA144" s="1" t="s">
         <v>130</v>
       </c>
@@ -14331,15 +14286,12 @@
       <c r="P145" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="S145" s="1"/>
-      <c r="T145" s="1"/>
       <c r="U145" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V145" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="W145" s="1"/>
       <c r="AA145" s="1" t="s">
         <v>130</v>
       </c>
@@ -14382,11 +14334,6 @@
       <c r="D146" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="S146" s="1"/>
-      <c r="T146" s="1"/>
-      <c r="U146" s="1"/>
-      <c r="V146" s="1"/>
-      <c r="W146" s="1"/>
     </row>
     <row r="147" spans="3:59" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C147" s="5" t="s">
@@ -14402,66 +14349,36 @@
       <c r="D148" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="S148" s="1"/>
-      <c r="T148" s="1"/>
-      <c r="U148" s="1"/>
-      <c r="V148" s="1"/>
-      <c r="W148" s="1"/>
     </row>
     <row r="149" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C149" s="9"/>
       <c r="D149" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="S149" s="1"/>
-      <c r="T149" s="1"/>
-      <c r="U149" s="1"/>
-      <c r="V149" s="1"/>
-      <c r="W149" s="1"/>
     </row>
     <row r="150" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C150" s="9"/>
       <c r="D150" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="S150" s="1"/>
-      <c r="T150" s="1"/>
-      <c r="U150" s="1"/>
-      <c r="V150" s="1"/>
-      <c r="W150" s="1"/>
     </row>
     <row r="151" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C151" s="9"/>
       <c r="D151" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="S151" s="1"/>
-      <c r="T151" s="1"/>
-      <c r="U151" s="1"/>
-      <c r="V151" s="1"/>
-      <c r="W151" s="1"/>
     </row>
     <row r="152" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C152" s="9"/>
       <c r="D152" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="S152" s="1"/>
-      <c r="T152" s="1"/>
-      <c r="U152" s="1"/>
-      <c r="V152" s="1"/>
-      <c r="W152" s="1"/>
     </row>
     <row r="153" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C153" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D153" s="10"/>
-      <c r="S153" s="1"/>
-      <c r="T153" s="1"/>
-      <c r="U153" s="1"/>
-      <c r="V153" s="1"/>
-      <c r="W153" s="1"/>
     </row>
     <row r="154" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C154" s="9"/>
@@ -14482,8 +14399,6 @@
         <v>86</v>
       </c>
       <c r="Q154"/>
-      <c r="S154" s="1"/>
-      <c r="T154" s="1"/>
       <c r="U154" s="1" t="s">
         <v>130</v>
       </c>
@@ -14553,8 +14468,6 @@
         <v>87</v>
       </c>
       <c r="Q155"/>
-      <c r="S155" s="1"/>
-      <c r="T155" s="1"/>
       <c r="U155" s="1" t="s">
         <v>130</v>
       </c>
@@ -14624,8 +14537,6 @@
         <v>88</v>
       </c>
       <c r="Q156"/>
-      <c r="S156" s="1"/>
-      <c r="T156" s="1"/>
       <c r="U156" s="1" t="s">
         <v>130</v>
       </c>
@@ -14695,8 +14606,6 @@
         <v>89</v>
       </c>
       <c r="Q157"/>
-      <c r="S157" s="1"/>
-      <c r="T157" s="1"/>
       <c r="U157" s="1" t="s">
         <v>130</v>
       </c>
@@ -14752,29 +14661,13 @@
       <c r="D158" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="S158" s="1"/>
-      <c r="T158" s="1"/>
-      <c r="U158" s="1"/>
-      <c r="V158" s="1"/>
-      <c r="W158" s="1"/>
-    </row>
-    <row r="159" spans="3:59" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="S159" s="1"/>
-      <c r="T159" s="1"/>
-      <c r="U159" s="1"/>
-      <c r="V159" s="1"/>
-      <c r="W159" s="1"/>
-    </row>
+    </row>
+    <row r="159" spans="3:59" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="160" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C160" s="4" t="s">
         <v>90</v>
       </c>
       <c r="D160" s="12"/>
-      <c r="S160" s="1"/>
-      <c r="T160" s="1"/>
-      <c r="U160" s="1"/>
-      <c r="V160" s="1"/>
-      <c r="W160" s="1"/>
     </row>
     <row r="161" spans="3:59" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C161" s="5" t="s">
@@ -14802,15 +14695,12 @@
       <c r="P162" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="S162" s="1"/>
-      <c r="T162" s="1"/>
       <c r="U162" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V162" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="W162" s="1"/>
       <c r="AA162" s="1" t="s">
         <v>130</v>
       </c>
@@ -14865,15 +14755,12 @@
       <c r="P163" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="S163" s="1"/>
-      <c r="T163" s="1"/>
       <c r="U163" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V163" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="W163" s="1"/>
       <c r="AA163" s="1" t="s">
         <v>130</v>
       </c>
@@ -14928,15 +14815,12 @@
       <c r="P164" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="S164" s="1"/>
-      <c r="T164" s="1"/>
       <c r="U164" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V164" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="W164" s="1"/>
       <c r="AA164" s="1" t="s">
         <v>130</v>
       </c>
@@ -14991,15 +14875,12 @@
       <c r="P165" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="S165" s="1"/>
-      <c r="T165" s="1"/>
       <c r="U165" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V165" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="W165" s="1"/>
       <c r="AA165" s="1" t="s">
         <v>130</v>
       </c>
@@ -15048,13 +14929,9 @@
       <c r="P166" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="S166" s="1"/>
-      <c r="T166" s="1"/>
-      <c r="U166" s="1"/>
       <c r="V166" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="W166" s="1"/>
       <c r="AB166" s="1" t="s">
         <v>95</v>
       </c>
@@ -15088,33 +14965,18 @@
       <c r="D168" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="S168" s="1"/>
-      <c r="T168" s="1"/>
-      <c r="U168" s="1"/>
-      <c r="V168" s="1"/>
-      <c r="W168" s="1"/>
     </row>
     <row r="169" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C169" s="9"/>
       <c r="D169" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="S169" s="1"/>
-      <c r="T169" s="1"/>
-      <c r="U169" s="1"/>
-      <c r="V169" s="1"/>
-      <c r="W169" s="1"/>
     </row>
     <row r="170" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C170" s="9"/>
       <c r="D170" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="S170" s="1"/>
-      <c r="T170" s="1"/>
-      <c r="U170" s="1"/>
-      <c r="V170" s="1"/>
-      <c r="W170" s="1"/>
     </row>
     <row r="171" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C171" s="17"/>
@@ -15122,7 +14984,7 @@
         <v>6</v>
       </c>
       <c r="E171" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F171">
         <v>1</v>
@@ -15131,16 +14993,16 @@
         <v>130</v>
       </c>
       <c r="H171" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J171" s="18"/>
       <c r="K171" s="32"/>
       <c r="L171" s="26"/>
       <c r="M171" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="N171">
         <v>1</v>
@@ -15149,13 +15011,13 @@
         <v>130</v>
       </c>
       <c r="P171" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="Q171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="S171" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="T171">
         <v>1</v>
@@ -15164,13 +15026,13 @@
         <v>130</v>
       </c>
       <c r="V171" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="W171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Y171" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="Z171">
         <v>1</v>
@@ -15179,13 +15041,13 @@
         <v>130</v>
       </c>
       <c r="AB171" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AC171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AE171" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AF171">
         <v>1</v>
@@ -15194,13 +15056,13 @@
         <v>130</v>
       </c>
       <c r="AH171" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AI171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AK171" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AL171">
         <v>1</v>
@@ -15209,13 +15071,13 @@
         <v>130</v>
       </c>
       <c r="AN171" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AO171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AQ171" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AR171">
         <v>1</v>
@@ -15224,13 +15086,13 @@
         <v>130</v>
       </c>
       <c r="AT171" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AU171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AW171" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AX171">
         <v>1</v>
@@ -15239,13 +15101,13 @@
         <v>130</v>
       </c>
       <c r="AZ171" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="BA171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="BC171" s="51" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="BD171">
         <v>1</v>
@@ -15254,10 +15116,10 @@
         <v>130</v>
       </c>
       <c r="BF171" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="BG171" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="172" spans="3:59" x14ac:dyDescent="0.2">
@@ -15265,11 +15127,6 @@
       <c r="D172" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="S172" s="1"/>
-      <c r="T172" s="1"/>
-      <c r="U172" s="1"/>
-      <c r="V172" s="1"/>
-      <c r="W172" s="1"/>
     </row>
     <row r="173" spans="3:59" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C173" s="5" t="s">
@@ -15297,15 +15154,12 @@
       <c r="P174" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="S174" s="1"/>
-      <c r="T174" s="1"/>
       <c r="U174" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V174" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="W174" s="1"/>
       <c r="AA174" s="1" t="s">
         <v>130</v>
       </c>
@@ -15360,15 +15214,12 @@
       <c r="P175" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S175" s="1"/>
-      <c r="T175" s="1"/>
       <c r="U175" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V175" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="W175" s="1"/>
       <c r="AA175" s="1" t="s">
         <v>130</v>
       </c>
@@ -15423,15 +15274,12 @@
       <c r="P176" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="S176" s="1"/>
-      <c r="T176" s="1"/>
       <c r="U176" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V176" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="W176" s="1"/>
       <c r="AA176" s="1" t="s">
         <v>130</v>
       </c>
@@ -15486,15 +15334,12 @@
       <c r="P177" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="S177" s="1"/>
-      <c r="T177" s="1"/>
       <c r="U177" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V177" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="W177" s="1"/>
       <c r="AA177" s="1" t="s">
         <v>130</v>
       </c>
@@ -15537,11 +15382,6 @@
       <c r="D178" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="S178" s="1"/>
-      <c r="T178" s="1"/>
-      <c r="U178" s="1"/>
-      <c r="V178" s="1"/>
-      <c r="W178" s="1"/>
     </row>
     <row r="179" spans="3:58" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C179" s="5" t="s">
@@ -15557,33 +15397,18 @@
       <c r="D180" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="S180" s="1"/>
-      <c r="T180" s="1"/>
-      <c r="U180" s="1"/>
-      <c r="V180" s="1"/>
-      <c r="W180" s="1"/>
     </row>
     <row r="181" spans="3:58" x14ac:dyDescent="0.2">
       <c r="C181" s="9"/>
       <c r="D181" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="S181" s="1"/>
-      <c r="T181" s="1"/>
-      <c r="U181" s="1"/>
-      <c r="V181" s="1"/>
-      <c r="W181" s="1"/>
     </row>
     <row r="182" spans="3:58" x14ac:dyDescent="0.2">
       <c r="C182" s="9"/>
       <c r="D182" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="S182" s="1"/>
-      <c r="T182" s="1"/>
-      <c r="U182" s="1"/>
-      <c r="V182" s="1"/>
-      <c r="W182" s="1"/>
     </row>
     <row r="183" spans="3:58" x14ac:dyDescent="0.2">
       <c r="C183" s="9"/>
@@ -15600,7 +15425,7 @@
         <v>130</v>
       </c>
       <c r="I183" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="M183" s="51" t="s">
         <v>139</v>
@@ -15612,7 +15437,7 @@
         <v>130</v>
       </c>
       <c r="Q183" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="S183" s="51" t="s">
         <v>139</v>
@@ -15623,9 +15448,8 @@
       <c r="U183" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="V183" s="1"/>
       <c r="W183" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="Y183" s="51" t="s">
         <v>139</v>
@@ -15687,11 +15511,6 @@
       <c r="D184" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="S184" s="1"/>
-      <c r="T184" s="1"/>
-      <c r="U184" s="1"/>
-      <c r="V184" s="1"/>
-      <c r="W184" s="1"/>
     </row>
     <row r="185" spans="3:58" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C185" s="5" t="s">
@@ -15719,15 +15538,12 @@
       <c r="P186" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="S186" s="1"/>
-      <c r="T186" s="1"/>
       <c r="U186" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V186" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="W186" s="1"/>
       <c r="AA186" s="1" t="s">
         <v>130</v>
       </c>
@@ -15782,15 +15598,12 @@
       <c r="P187" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="S187" s="1"/>
-      <c r="T187" s="1"/>
       <c r="U187" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V187" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="W187" s="1"/>
       <c r="AA187" s="1" t="s">
         <v>130</v>
       </c>
@@ -15845,15 +15658,12 @@
       <c r="P188" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="S188" s="1"/>
-      <c r="T188" s="1"/>
       <c r="U188" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V188" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="W188" s="1"/>
       <c r="AA188" s="1" t="s">
         <v>130</v>
       </c>
@@ -15908,15 +15718,12 @@
       <c r="P189" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="S189" s="1"/>
-      <c r="T189" s="1"/>
       <c r="U189" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V189" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="W189" s="1"/>
       <c r="AA189" s="1" t="s">
         <v>130</v>
       </c>
@@ -15971,15 +15778,12 @@
       <c r="P190" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="S190" s="1"/>
-      <c r="T190" s="1"/>
       <c r="U190" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V190" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="W190" s="1"/>
       <c r="AA190" s="1" t="s">
         <v>130</v>
       </c>
@@ -16043,15 +15847,12 @@
       <c r="P192" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="S192" s="1"/>
-      <c r="T192" s="1"/>
       <c r="U192" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V192" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="W192" s="1"/>
       <c r="AA192" s="1" t="s">
         <v>130</v>
       </c>
@@ -16106,15 +15907,12 @@
       <c r="P193" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="S193" s="1"/>
-      <c r="T193" s="1"/>
       <c r="U193" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V193" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="W193" s="1"/>
       <c r="AA193" s="1" t="s">
         <v>130</v>
       </c>
@@ -16169,15 +15967,12 @@
       <c r="P194" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="S194" s="1"/>
-      <c r="T194" s="1"/>
       <c r="U194" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V194" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="W194" s="1"/>
       <c r="AA194" s="1" t="s">
         <v>130</v>
       </c>
@@ -16232,15 +16027,12 @@
       <c r="P195" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="S195" s="1"/>
-      <c r="T195" s="1"/>
       <c r="U195" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V195" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="W195" s="1"/>
       <c r="AA195" s="1" t="s">
         <v>130</v>
       </c>
@@ -16295,15 +16087,12 @@
       <c r="P196" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="S196" s="1"/>
-      <c r="T196" s="1"/>
       <c r="U196" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V196" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="W196" s="1"/>
       <c r="AA196" s="1" t="s">
         <v>130</v>
       </c>
@@ -16355,66 +16144,36 @@
       <c r="D198" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="S198" s="1"/>
-      <c r="T198" s="1"/>
-      <c r="U198" s="1"/>
-      <c r="V198" s="1"/>
-      <c r="W198" s="1"/>
     </row>
     <row r="199" spans="2:59" x14ac:dyDescent="0.2">
       <c r="C199" s="9"/>
       <c r="D199" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="S199" s="1"/>
-      <c r="T199" s="1"/>
-      <c r="U199" s="1"/>
-      <c r="V199" s="1"/>
-      <c r="W199" s="1"/>
     </row>
     <row r="200" spans="2:59" x14ac:dyDescent="0.2">
       <c r="C200" s="9"/>
       <c r="D200" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="S200" s="1"/>
-      <c r="T200" s="1"/>
-      <c r="U200" s="1"/>
-      <c r="V200" s="1"/>
-      <c r="W200" s="1"/>
     </row>
     <row r="201" spans="2:59" x14ac:dyDescent="0.2">
       <c r="C201" s="9"/>
       <c r="D201" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="S201" s="1"/>
-      <c r="T201" s="1"/>
-      <c r="U201" s="1"/>
-      <c r="V201" s="1"/>
-      <c r="W201" s="1"/>
     </row>
     <row r="202" spans="2:59" x14ac:dyDescent="0.2">
       <c r="C202" s="9"/>
       <c r="D202" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="S202" s="1"/>
-      <c r="T202" s="1"/>
-      <c r="U202" s="1"/>
-      <c r="V202" s="1"/>
-      <c r="W202" s="1"/>
     </row>
     <row r="203" spans="2:59" x14ac:dyDescent="0.2">
       <c r="C203" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D203" s="10"/>
-      <c r="S203" s="1"/>
-      <c r="T203" s="1"/>
-      <c r="U203" s="1"/>
-      <c r="V203" s="1"/>
-      <c r="W203" s="1"/>
     </row>
     <row r="204" spans="2:59" x14ac:dyDescent="0.2">
       <c r="C204" s="9"/>
@@ -16530,8 +16289,8 @@
         <v>110</v>
       </c>
       <c r="AC205"/>
-      <c r="AE205" s="60"/>
-      <c r="AF205" s="60"/>
+      <c r="AE205" s="1"/>
+      <c r="AF205" s="1"/>
       <c r="AG205" s="1" t="s">
         <v>130</v>
       </c>
@@ -16539,7 +16298,7 @@
         <v>110</v>
       </c>
       <c r="AI205"/>
-      <c r="AJ205" s="60"/>
+      <c r="AJ205" s="1"/>
       <c r="AK205" s="1"/>
       <c r="AL205" s="1"/>
       <c r="AM205" s="1" t="s">
@@ -16614,8 +16373,8 @@
         <v>111</v>
       </c>
       <c r="AC206"/>
-      <c r="AE206" s="60"/>
-      <c r="AF206" s="60"/>
+      <c r="AE206" s="1"/>
+      <c r="AF206" s="1"/>
       <c r="AG206" s="1" t="s">
         <v>130</v>
       </c>
@@ -16623,7 +16382,7 @@
         <v>111</v>
       </c>
       <c r="AI206"/>
-      <c r="AJ206" s="60"/>
+      <c r="AJ206" s="1"/>
       <c r="AK206" s="1"/>
       <c r="AL206" s="1"/>
       <c r="AM206" s="1" t="s">
@@ -16698,8 +16457,8 @@
         <v>112</v>
       </c>
       <c r="AC207"/>
-      <c r="AE207" s="60"/>
-      <c r="AF207" s="60"/>
+      <c r="AE207" s="1"/>
+      <c r="AF207" s="1"/>
       <c r="AG207" s="1" t="s">
         <v>130</v>
       </c>
@@ -16707,7 +16466,7 @@
         <v>112</v>
       </c>
       <c r="AI207"/>
-      <c r="AJ207" s="60"/>
+      <c r="AJ207" s="1"/>
       <c r="AK207" s="1"/>
       <c r="AL207" s="1"/>
       <c r="AM207" s="1" t="s">
@@ -16766,12 +16525,12 @@
       <c r="AA208" s="1"/>
       <c r="AB208" s="1"/>
       <c r="AC208" s="1"/>
-      <c r="AE208" s="60"/>
-      <c r="AF208" s="60"/>
+      <c r="AE208" s="1"/>
+      <c r="AF208" s="1"/>
       <c r="AG208" s="1"/>
       <c r="AH208" s="1"/>
       <c r="AI208" s="1"/>
-      <c r="AJ208" s="60"/>
+      <c r="AJ208" s="1"/>
       <c r="AK208" s="1"/>
       <c r="AL208" s="1"/>
       <c r="AM208" s="1"/>
@@ -16794,9 +16553,6 @@
       <c r="C209" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="U209" s="1"/>
-      <c r="V209" s="1"/>
-      <c r="W209" s="1"/>
     </row>
     <row r="210" spans="3:59" x14ac:dyDescent="0.2">
       <c r="D210" s="11" t="s">
@@ -16823,14 +16579,14 @@
         <v>130</v>
       </c>
       <c r="V210" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="W210"/>
       <c r="AA210" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AB210" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AC210"/>
       <c r="AG210" s="1" t="s">
@@ -16893,14 +16649,14 @@
         <v>130</v>
       </c>
       <c r="V211" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="W211"/>
       <c r="AA211" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AB211" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AC211"/>
       <c r="AG211" s="1" t="s">
@@ -16964,14 +16720,14 @@
         <v>130</v>
       </c>
       <c r="V212" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="W212"/>
       <c r="AA212" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AB212" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AC212"/>
       <c r="AG212" s="1" t="s">
@@ -17035,14 +16791,14 @@
         <v>130</v>
       </c>
       <c r="V213" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="W213"/>
       <c r="AA213" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AB213" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AC213"/>
       <c r="AG213" s="1" t="s">
@@ -17085,161 +16841,147 @@
       <c r="D214" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="U214" s="1"/>
-      <c r="V214" s="1"/>
-      <c r="W214" s="1"/>
       <c r="AN214" s="2"/>
-      <c r="AO214" s="60"/>
       <c r="BG214"/>
     </row>
     <row r="215" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C215" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="U215" s="1"/>
-      <c r="V215" s="1"/>
-      <c r="W215" s="1"/>
       <c r="AN215" s="2"/>
-      <c r="AO215" s="60"/>
     </row>
     <row r="216" spans="3:59" x14ac:dyDescent="0.2">
       <c r="D216" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E216" s="1" t="s">
+      <c r="G216" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="H216" t="s">
         <v>184</v>
-      </c>
-      <c r="G216" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H216" t="s">
-        <v>185</v>
       </c>
       <c r="I216"/>
       <c r="O216" s="1" t="s">
         <v>130</v>
       </c>
       <c r="P216" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="Q216"/>
       <c r="U216" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V216" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="W216"/>
       <c r="AA216" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AB216" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AC216"/>
       <c r="AG216" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AH216" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AI216"/>
       <c r="AM216" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AN216" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AO216"/>
       <c r="AS216" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AT216" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AU216"/>
       <c r="AY216" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AZ216" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="BA216"/>
       <c r="BE216" s="1" t="s">
         <v>130</v>
       </c>
       <c r="BF216" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="217" spans="3:59" x14ac:dyDescent="0.2">
       <c r="D217" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E217" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="G217" s="1" t="s">
         <v>130</v>
       </c>
       <c r="H217" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I217"/>
       <c r="O217" s="1" t="s">
         <v>130</v>
       </c>
       <c r="P217" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="Q217"/>
       <c r="U217" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V217" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="W217"/>
       <c r="AA217" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AB217" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AC217"/>
       <c r="AG217" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AH217" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AI217"/>
       <c r="AM217" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AN217" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AO217"/>
       <c r="AS217" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AT217" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AU217"/>
       <c r="AY217" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AZ217" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="BA217"/>
       <c r="BE217" s="1" t="s">
         <v>130</v>
       </c>
       <c r="BF217" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="BG217"/>
     </row>
@@ -17247,70 +16989,67 @@
       <c r="D218" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="E218" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="G218" s="1" t="s">
         <v>130</v>
       </c>
       <c r="H218" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I218"/>
       <c r="O218" s="1" t="s">
         <v>130</v>
       </c>
       <c r="P218" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Q218"/>
       <c r="U218" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V218" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="W218"/>
       <c r="AA218" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AB218" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AC218"/>
       <c r="AG218" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AH218" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AI218"/>
       <c r="AM218" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AN218" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AO218"/>
       <c r="AS218" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AT218" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AU218"/>
       <c r="AY218" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AZ218" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="BA218"/>
       <c r="BE218" s="1" t="s">
         <v>130</v>
       </c>
       <c r="BF218" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="BG218"/>
     </row>
@@ -17318,70 +17057,67 @@
       <c r="D219" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E219" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="G219" s="1" t="s">
         <v>130</v>
       </c>
       <c r="H219" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I219"/>
       <c r="O219" s="1" t="s">
         <v>130</v>
       </c>
       <c r="P219" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="Q219"/>
       <c r="U219" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V219" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="W219"/>
       <c r="AA219" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AB219" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AC219"/>
       <c r="AG219" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AH219" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AI219"/>
       <c r="AM219" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AN219" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AO219"/>
       <c r="AS219" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AT219" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="AU219"/>
       <c r="AY219" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AZ219" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="BA219"/>
       <c r="BE219" s="1" t="s">
         <v>130</v>
       </c>
       <c r="BF219" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="BG219"/>
     </row>
@@ -17396,11 +17132,8 @@
     </row>
     <row r="221" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C221" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="U221" s="1"/>
-      <c r="V221" s="1"/>
-      <c r="W221" s="1"/>
+        <v>252</v>
+      </c>
     </row>
     <row r="222" spans="3:59" x14ac:dyDescent="0.2">
       <c r="D222" s="11" t="s">
@@ -17410,7 +17143,6 @@
       <c r="I222"/>
       <c r="P222"/>
       <c r="Q222"/>
-      <c r="U222" s="1"/>
       <c r="V222"/>
       <c r="W222"/>
       <c r="AB222"/>
@@ -17430,7 +17162,6 @@
       <c r="I223"/>
       <c r="P223"/>
       <c r="Q223"/>
-      <c r="U223" s="1"/>
       <c r="V223"/>
       <c r="W223"/>
       <c r="AB223"/>
@@ -17454,7 +17185,6 @@
       <c r="I224"/>
       <c r="P224"/>
       <c r="Q224"/>
-      <c r="U224" s="1"/>
       <c r="V224"/>
       <c r="W224"/>
       <c r="AB224"/>
@@ -17478,93 +17208,89 @@
         <v>130</v>
       </c>
       <c r="H225" t="s">
-        <v>262</v>
-      </c>
-      <c r="I225" s="63" t="s">
-        <v>256</v>
+        <v>261</v>
+      </c>
+      <c r="I225" s="1" t="s">
+        <v>255</v>
       </c>
       <c r="O225" s="1" t="s">
         <v>130</v>
       </c>
       <c r="P225" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="Q225" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="U225" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V225" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="W225" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AA225" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AB225" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="AC225" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AG225" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AH225" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AI225" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AM225" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AN225" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AO225" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AS225" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AT225" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AU225" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AY225" s="1" t="s">
         <v>130</v>
       </c>
       <c r="AZ225" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="BA225" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="BE225" s="1" t="s">
         <v>130</v>
       </c>
       <c r="BF225" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="BG225" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="226" spans="3:59" x14ac:dyDescent="0.2">
       <c r="D226" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="U226" s="1"/>
-      <c r="V226" s="1"/>
-      <c r="W226" s="1"/>
       <c r="AN226" s="2"/>
-      <c r="AO226" s="60"/>
       <c r="AZ226"/>
       <c r="BA226"/>
       <c r="BF226"/>
@@ -17572,13 +17298,9 @@
     </row>
     <row r="227" spans="3:59" x14ac:dyDescent="0.2">
       <c r="C227" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="U227" s="1"/>
-      <c r="V227" s="1"/>
-      <c r="W227" s="1"/>
+        <v>253</v>
+      </c>
       <c r="AN227" s="2"/>
-      <c r="AO227" s="60"/>
     </row>
     <row r="228" spans="3:59" x14ac:dyDescent="0.2">
       <c r="D228" s="11" t="s">
@@ -17588,7 +17310,6 @@
       <c r="I228"/>
       <c r="P228"/>
       <c r="Q228"/>
-      <c r="U228" s="1"/>
       <c r="V228"/>
       <c r="W228"/>
       <c r="AB228"/>
@@ -17611,7 +17332,6 @@
       <c r="I229"/>
       <c r="P229"/>
       <c r="Q229"/>
-      <c r="U229" s="1"/>
       <c r="V229"/>
       <c r="W229"/>
       <c r="AB229"/>
@@ -17635,7 +17355,6 @@
       <c r="I230"/>
       <c r="P230"/>
       <c r="Q230"/>
-      <c r="U230" s="1"/>
       <c r="V230"/>
       <c r="W230"/>
       <c r="AB230"/>
@@ -17655,89 +17374,86 @@
       <c r="D231" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E231" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="G231" s="1" t="s">
         <v>130</v>
       </c>
       <c r="H231" t="s">
+        <v>262</v>
+      </c>
+      <c r="I231" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="O231" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="P231" t="s">
         <v>263</v>
       </c>
-      <c r="I231" s="63" t="s">
-        <v>256</v>
-      </c>
-      <c r="O231" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="P231" t="s">
-        <v>264</v>
-      </c>
       <c r="Q231" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="U231" s="1" t="s">
         <v>130</v>
       </c>
       <c r="V231" t="s">
+        <v>265</v>
+      </c>
+      <c r="W231" t="s">
+        <v>255</v>
+      </c>
+      <c r="AA231" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AB231" t="s">
+        <v>265</v>
+      </c>
+      <c r="AC231" t="s">
+        <v>255</v>
+      </c>
+      <c r="AG231" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AH231" t="s">
         <v>266</v>
       </c>
-      <c r="W231" t="s">
-        <v>256</v>
-      </c>
-      <c r="AA231" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="AB231" t="s">
-        <v>266</v>
-      </c>
-      <c r="AC231" t="s">
-        <v>256</v>
-      </c>
-      <c r="AG231" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="AH231" t="s">
+      <c r="AI231" t="s">
+        <v>255</v>
+      </c>
+      <c r="AM231" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AN231" t="s">
         <v>267</v>
       </c>
-      <c r="AI231" t="s">
-        <v>256</v>
-      </c>
-      <c r="AM231" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="AN231" t="s">
+      <c r="AO231" t="s">
+        <v>255</v>
+      </c>
+      <c r="AS231" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AT231" t="s">
         <v>268</v>
       </c>
-      <c r="AO231" t="s">
-        <v>256</v>
-      </c>
-      <c r="AS231" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="AT231" t="s">
+      <c r="AU231" t="s">
+        <v>255</v>
+      </c>
+      <c r="AY231" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AZ231" t="s">
+        <v>262</v>
+      </c>
+      <c r="BA231" t="s">
+        <v>255</v>
+      </c>
+      <c r="BE231" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="BF231" t="s">
         <v>269</v>
       </c>
-      <c r="AU231" t="s">
-        <v>256</v>
-      </c>
-      <c r="AY231" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="AZ231" t="s">
-        <v>263</v>
-      </c>
-      <c r="BA231" t="s">
-        <v>256</v>
-      </c>
-      <c r="BE231" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="BF231" t="s">
-        <v>270</v>
-      </c>
       <c r="BG231" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="232" spans="3:59" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
added multi temperature to scatter plots and box plots
and added scatter plot of two variables to L2
</commit_message>
<xml_diff>
--- a/scratch/FormattedCutTableL3_template_md.xlsx
+++ b/scratch/FormattedCutTableL3_template_md.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/sam mac stove data/DOE Data/lab tests/5 stoves comparison/all stoves/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C03A435-CFB4-8B44-B06C-6A7B85305270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{872F99AA-3B61-2947-8205-B24BEE64E507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3640" yWindow="2960" windowWidth="27200" windowHeight="14860" xr2:uid="{1837E1AF-DB18-D64C-9443-79C0B4F568AD}"/>
+    <workbookView xWindow="2400" yWindow="2680" windowWidth="27200" windowHeight="14860" xr2:uid="{1837E1AF-DB18-D64C-9443-79C0B4F568AD}"/>
   </bookViews>
   <sheets>
     <sheet name="all data expanded" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3656" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3959" uniqueCount="302">
   <si>
     <t>Metrics</t>
   </si>
@@ -938,6 +938,9 @@
   </si>
   <si>
     <t>Control Temperature, LP Gasifier</t>
+  </si>
+  <si>
+    <t>0B</t>
   </si>
 </sst>
 </file>
@@ -1745,7 +1748,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A22C1804-EB7C-BF43-9073-75DDFAF0ED4D}">
-  <dimension ref="B1:BS238"/>
+  <dimension ref="B1:BY238"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" style="1" customWidth="1"/>
@@ -1782,10 +1785,12 @@
     <col min="58" max="58" width="14" style="1" customWidth="1"/>
     <col min="59" max="64" width="10.83203125" style="1"/>
     <col min="65" max="70" width="8.6640625" style="1" customWidth="1"/>
-    <col min="71" max="16384" width="10.83203125" style="1"/>
+    <col min="71" max="71" width="10.83203125" style="1"/>
+    <col min="72" max="76" width="8.6640625" style="1" customWidth="1"/>
+    <col min="77" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:71" ht="34" x14ac:dyDescent="0.2">
+    <row r="1" spans="3:77" ht="34" x14ac:dyDescent="0.2">
       <c r="K1" s="17" t="s">
         <v>163</v>
       </c>
@@ -1849,8 +1854,16 @@
       <c r="BS1" s="58" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="2" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT1" s="17"/>
+      <c r="BU1" s="17"/>
+      <c r="BV1" s="17"/>
+      <c r="BW1" s="17"/>
+      <c r="BX1" s="17"/>
+      <c r="BY1" s="58" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="2" spans="3:77" x14ac:dyDescent="0.2">
       <c r="K2" s="17" t="s">
         <v>166</v>
       </c>
@@ -1914,8 +1927,16 @@
       <c r="BS2" s="17" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="3" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT2" s="17"/>
+      <c r="BU2" s="17"/>
+      <c r="BV2" s="17"/>
+      <c r="BW2" s="17"/>
+      <c r="BX2" s="17"/>
+      <c r="BY2" s="17">
+        <v>2520</v>
+      </c>
+    </row>
+    <row r="3" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C3" s="14" t="s">
         <v>0</v>
       </c>
@@ -2121,8 +2142,26 @@
       <c r="BS3" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="4" spans="3:71" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="BT3" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="BU3" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="BV3" s="15" t="s">
+        <v>275</v>
+      </c>
+      <c r="BW3" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="BX3" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="BY3" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="4" spans="3:77" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C4" s="17"/>
       <c r="D4"/>
       <c r="E4"/>
@@ -2206,8 +2245,15 @@
         <v>113</v>
       </c>
       <c r="BR4"/>
-    </row>
-    <row r="5" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT4"/>
+      <c r="BU4"/>
+      <c r="BV4"/>
+      <c r="BW4" t="s">
+        <v>113</v>
+      </c>
+      <c r="BX4"/>
+    </row>
+    <row r="5" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C5" s="19" t="s">
         <v>1</v>
       </c>
@@ -2271,8 +2317,13 @@
       <c r="BP5"/>
       <c r="BQ5"/>
       <c r="BR5"/>
-    </row>
-    <row r="6" spans="3:71" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT5"/>
+      <c r="BU5"/>
+      <c r="BV5"/>
+      <c r="BW5"/>
+      <c r="BX5"/>
+    </row>
+    <row r="6" spans="3:77" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C6" s="21" t="s">
         <v>2</v>
       </c>
@@ -2337,8 +2388,13 @@
       <c r="BP6" s="23"/>
       <c r="BQ6" s="23"/>
       <c r="BR6" s="29"/>
-    </row>
-    <row r="7" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT6" s="50"/>
+      <c r="BU6" s="23"/>
+      <c r="BV6" s="23"/>
+      <c r="BW6" s="23"/>
+      <c r="BX6" s="29"/>
+    </row>
+    <row r="7" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C7" s="17"/>
       <c r="D7" s="25" t="s">
         <v>3</v>
@@ -2468,8 +2524,19 @@
         <v>15</v>
       </c>
       <c r="BR7"/>
-    </row>
-    <row r="8" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT7" s="51"/>
+      <c r="BU7">
+        <v>0</v>
+      </c>
+      <c r="BV7" t="s">
+        <v>128</v>
+      </c>
+      <c r="BW7" t="s">
+        <v>15</v>
+      </c>
+      <c r="BX7"/>
+    </row>
+    <row r="8" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C8" s="17"/>
       <c r="D8" s="25" t="s">
         <v>4</v>
@@ -2599,8 +2666,19 @@
         <v>16</v>
       </c>
       <c r="BR8"/>
-    </row>
-    <row r="9" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT8" s="51"/>
+      <c r="BU8">
+        <v>0</v>
+      </c>
+      <c r="BV8" t="s">
+        <v>128</v>
+      </c>
+      <c r="BW8" t="s">
+        <v>16</v>
+      </c>
+      <c r="BX8"/>
+    </row>
+    <row r="9" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C9" s="17"/>
       <c r="D9" s="25" t="s">
         <v>5</v>
@@ -2730,8 +2808,19 @@
         <v>17</v>
       </c>
       <c r="BR9"/>
-    </row>
-    <row r="10" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT9" s="51"/>
+      <c r="BU9">
+        <v>0</v>
+      </c>
+      <c r="BV9" t="s">
+        <v>128</v>
+      </c>
+      <c r="BW9" t="s">
+        <v>17</v>
+      </c>
+      <c r="BX9"/>
+    </row>
+    <row r="10" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C10" s="17"/>
       <c r="D10" s="25" t="s">
         <v>6</v>
@@ -2861,8 +2950,19 @@
         <v>18</v>
       </c>
       <c r="BR10"/>
-    </row>
-    <row r="11" spans="3:71" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT10" s="51"/>
+      <c r="BU10">
+        <v>0</v>
+      </c>
+      <c r="BV10" t="s">
+        <v>128</v>
+      </c>
+      <c r="BW10" t="s">
+        <v>18</v>
+      </c>
+      <c r="BX10"/>
+    </row>
+    <row r="11" spans="3:77" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C11" s="27" t="s">
         <v>7</v>
       </c>
@@ -2927,8 +3027,13 @@
       <c r="BP11" s="29"/>
       <c r="BQ11" s="29"/>
       <c r="BR11" s="29"/>
-    </row>
-    <row r="12" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT11" s="52"/>
+      <c r="BU11" s="29"/>
+      <c r="BV11" s="29"/>
+      <c r="BW11" s="29"/>
+      <c r="BX11" s="29"/>
+    </row>
+    <row r="12" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C12" s="17"/>
       <c r="D12" s="25" t="s">
         <v>3</v>
@@ -2992,8 +3097,13 @@
       <c r="BP12"/>
       <c r="BQ12"/>
       <c r="BR12"/>
-    </row>
-    <row r="13" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT12" s="51"/>
+      <c r="BU12"/>
+      <c r="BV12"/>
+      <c r="BW12"/>
+      <c r="BX12"/>
+    </row>
+    <row r="13" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C13" s="17"/>
       <c r="D13" s="25" t="s">
         <v>4</v>
@@ -3057,8 +3167,13 @@
       <c r="BP13"/>
       <c r="BQ13"/>
       <c r="BR13"/>
-    </row>
-    <row r="14" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT13" s="51"/>
+      <c r="BU13"/>
+      <c r="BV13"/>
+      <c r="BW13"/>
+      <c r="BX13"/>
+    </row>
+    <row r="14" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C14" s="17"/>
       <c r="D14" s="25" t="s">
         <v>5</v>
@@ -3122,8 +3237,13 @@
       <c r="BP14"/>
       <c r="BQ14"/>
       <c r="BR14"/>
-    </row>
-    <row r="15" spans="3:71" x14ac:dyDescent="0.2">
+      <c r="BT14" s="51"/>
+      <c r="BU14"/>
+      <c r="BV14"/>
+      <c r="BW14"/>
+      <c r="BX14"/>
+    </row>
+    <row r="15" spans="3:77" x14ac:dyDescent="0.2">
       <c r="C15" s="17"/>
       <c r="D15" s="25" t="s">
         <v>6</v>
@@ -3187,8 +3307,13 @@
       <c r="BP15"/>
       <c r="BQ15"/>
       <c r="BR15"/>
-    </row>
-    <row r="16" spans="3:71" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT15" s="51"/>
+      <c r="BU15"/>
+      <c r="BV15"/>
+      <c r="BW15"/>
+      <c r="BX15"/>
+    </row>
+    <row r="16" spans="3:77" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C16" s="27" t="s">
         <v>8</v>
       </c>
@@ -3253,8 +3378,13 @@
       <c r="BP16" s="29"/>
       <c r="BQ16" s="29"/>
       <c r="BR16" s="29"/>
-    </row>
-    <row r="17" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT16" s="52"/>
+      <c r="BU16" s="29"/>
+      <c r="BV16" s="29"/>
+      <c r="BW16" s="29"/>
+      <c r="BX16" s="29"/>
+    </row>
+    <row r="17" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C17" s="17"/>
       <c r="D17" s="25" t="s">
         <v>3</v>
@@ -3384,8 +3514,19 @@
         <v>9</v>
       </c>
       <c r="BR17"/>
-    </row>
-    <row r="18" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT17" s="51"/>
+      <c r="BU17">
+        <v>1</v>
+      </c>
+      <c r="BV17" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW17" t="s">
+        <v>9</v>
+      </c>
+      <c r="BX17"/>
+    </row>
+    <row r="18" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C18" s="17"/>
       <c r="D18" s="25" t="s">
         <v>4</v>
@@ -3515,8 +3656,19 @@
         <v>10</v>
       </c>
       <c r="BR18"/>
-    </row>
-    <row r="19" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT18" s="51"/>
+      <c r="BU18">
+        <v>1</v>
+      </c>
+      <c r="BV18" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW18" t="s">
+        <v>10</v>
+      </c>
+      <c r="BX18"/>
+    </row>
+    <row r="19" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C19" s="17"/>
       <c r="D19" s="25" t="s">
         <v>5</v>
@@ -3646,8 +3798,19 @@
         <v>11</v>
       </c>
       <c r="BR19"/>
-    </row>
-    <row r="20" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT19" s="51"/>
+      <c r="BU19">
+        <v>1</v>
+      </c>
+      <c r="BV19" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW19" t="s">
+        <v>11</v>
+      </c>
+      <c r="BX19"/>
+    </row>
+    <row r="20" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C20" s="17"/>
       <c r="D20" s="25" t="s">
         <v>6</v>
@@ -3777,8 +3940,19 @@
         <v>12</v>
       </c>
       <c r="BR20"/>
-    </row>
-    <row r="21" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT20" s="51"/>
+      <c r="BU20">
+        <v>1</v>
+      </c>
+      <c r="BV20" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW20" t="s">
+        <v>12</v>
+      </c>
+      <c r="BX20"/>
+    </row>
+    <row r="21" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C21" s="17"/>
       <c r="D21" s="25" t="s">
         <v>13</v>
@@ -3908,8 +4082,19 @@
         <v>14</v>
       </c>
       <c r="BR21"/>
-    </row>
-    <row r="22" spans="3:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT21" s="51"/>
+      <c r="BU21">
+        <v>1</v>
+      </c>
+      <c r="BV21" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW21" t="s">
+        <v>14</v>
+      </c>
+      <c r="BX21"/>
+    </row>
+    <row r="22" spans="3:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C22" s="27" t="s">
         <v>139</v>
       </c>
@@ -3974,8 +4159,13 @@
       <c r="BP22" s="29"/>
       <c r="BQ22" s="29"/>
       <c r="BR22" s="29"/>
-    </row>
-    <row r="23" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT22" s="52"/>
+      <c r="BU22" s="29"/>
+      <c r="BV22" s="29"/>
+      <c r="BW22" s="29"/>
+      <c r="BX22" s="29"/>
+    </row>
+    <row r="23" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C23" s="17"/>
       <c r="D23" s="25" t="s">
         <v>3</v>
@@ -4127,8 +4317,21 @@
         <v>15</v>
       </c>
       <c r="BR23"/>
-    </row>
-    <row r="24" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT23" s="51" t="s">
+        <v>137</v>
+      </c>
+      <c r="BU23">
+        <v>1</v>
+      </c>
+      <c r="BV23" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW23" t="s">
+        <v>15</v>
+      </c>
+      <c r="BX23"/>
+    </row>
+    <row r="24" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C24" s="17"/>
       <c r="D24" s="25" t="s">
         <v>4</v>
@@ -4280,8 +4483,21 @@
         <v>16</v>
       </c>
       <c r="BR24"/>
-    </row>
-    <row r="25" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT24" s="51" t="s">
+        <v>137</v>
+      </c>
+      <c r="BU24">
+        <v>1</v>
+      </c>
+      <c r="BV24" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW24" t="s">
+        <v>16</v>
+      </c>
+      <c r="BX24"/>
+    </row>
+    <row r="25" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C25" s="17"/>
       <c r="D25" s="25" t="s">
         <v>5</v>
@@ -4433,8 +4649,21 @@
         <v>17</v>
       </c>
       <c r="BR25"/>
-    </row>
-    <row r="26" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT25" s="51" t="s">
+        <v>137</v>
+      </c>
+      <c r="BU25">
+        <v>1</v>
+      </c>
+      <c r="BV25" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW25" t="s">
+        <v>17</v>
+      </c>
+      <c r="BX25"/>
+    </row>
+    <row r="26" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C26" s="17"/>
       <c r="D26" s="25" t="s">
         <v>6</v>
@@ -4586,8 +4815,21 @@
         <v>18</v>
       </c>
       <c r="BR26"/>
-    </row>
-    <row r="27" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT26" s="51" t="s">
+        <v>137</v>
+      </c>
+      <c r="BU26">
+        <v>1</v>
+      </c>
+      <c r="BV26" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW26" t="s">
+        <v>18</v>
+      </c>
+      <c r="BX26"/>
+    </row>
+    <row r="27" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C27" s="17"/>
       <c r="D27" s="25" t="s">
         <v>13</v>
@@ -4685,8 +4927,17 @@
       </c>
       <c r="BQ27"/>
       <c r="BR27"/>
-    </row>
-    <row r="28" spans="3:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT27" s="51"/>
+      <c r="BU27">
+        <v>1</v>
+      </c>
+      <c r="BV27" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW27"/>
+      <c r="BX27"/>
+    </row>
+    <row r="28" spans="3:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C28" s="27" t="s">
         <v>19</v>
       </c>
@@ -4751,8 +5002,13 @@
       <c r="BP28" s="29"/>
       <c r="BQ28" s="29"/>
       <c r="BR28" s="29"/>
-    </row>
-    <row r="29" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT28" s="52"/>
+      <c r="BU28" s="29"/>
+      <c r="BV28" s="29"/>
+      <c r="BW28" s="29"/>
+      <c r="BX28" s="29"/>
+    </row>
+    <row r="29" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C29" s="17"/>
       <c r="D29" s="25" t="s">
         <v>3</v>
@@ -4882,8 +5138,19 @@
         <v>20</v>
       </c>
       <c r="BR29"/>
-    </row>
-    <row r="30" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT29" s="51"/>
+      <c r="BU29">
+        <v>1</v>
+      </c>
+      <c r="BV29" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW29" t="s">
+        <v>20</v>
+      </c>
+      <c r="BX29"/>
+    </row>
+    <row r="30" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C30" s="17"/>
       <c r="D30" s="25" t="s">
         <v>4</v>
@@ -5013,8 +5280,19 @@
         <v>21</v>
       </c>
       <c r="BR30"/>
-    </row>
-    <row r="31" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT30" s="51"/>
+      <c r="BU30">
+        <v>1</v>
+      </c>
+      <c r="BV30" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW30" t="s">
+        <v>21</v>
+      </c>
+      <c r="BX30"/>
+    </row>
+    <row r="31" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C31" s="17"/>
       <c r="D31" s="25" t="s">
         <v>5</v>
@@ -5144,8 +5422,19 @@
         <v>22</v>
       </c>
       <c r="BR31"/>
-    </row>
-    <row r="32" spans="3:70" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="BT31" s="51"/>
+      <c r="BU31">
+        <v>1</v>
+      </c>
+      <c r="BV31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW31" t="s">
+        <v>22</v>
+      </c>
+      <c r="BX31"/>
+    </row>
+    <row r="32" spans="3:76" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C32" s="34"/>
       <c r="D32" s="35" t="s">
         <v>6</v>
@@ -5275,8 +5564,19 @@
         <v>23</v>
       </c>
       <c r="BR32"/>
-    </row>
-    <row r="33" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT32" s="51"/>
+      <c r="BU32">
+        <v>1</v>
+      </c>
+      <c r="BV32" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW32" t="s">
+        <v>23</v>
+      </c>
+      <c r="BX32"/>
+    </row>
+    <row r="33" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C33" s="27" t="s">
         <v>119</v>
       </c>
@@ -5340,8 +5640,13 @@
       <c r="BP33" s="29"/>
       <c r="BQ33" s="29"/>
       <c r="BR33"/>
-    </row>
-    <row r="34" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT33" s="52"/>
+      <c r="BU33" s="29"/>
+      <c r="BV33" s="29"/>
+      <c r="BW33" s="29"/>
+      <c r="BX33"/>
+    </row>
+    <row r="34" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C34" s="17"/>
       <c r="D34" s="25" t="s">
         <v>3</v>
@@ -5471,8 +5776,19 @@
         <v>120</v>
       </c>
       <c r="BR34"/>
-    </row>
-    <row r="35" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT34" s="51"/>
+      <c r="BU34">
+        <v>1</v>
+      </c>
+      <c r="BV34" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW34" t="s">
+        <v>120</v>
+      </c>
+      <c r="BX34"/>
+    </row>
+    <row r="35" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C35" s="17"/>
       <c r="D35" s="25" t="s">
         <v>4</v>
@@ -5602,8 +5918,19 @@
         <v>121</v>
       </c>
       <c r="BR35"/>
-    </row>
-    <row r="36" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT35" s="51"/>
+      <c r="BU35">
+        <v>1</v>
+      </c>
+      <c r="BV35" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW35" t="s">
+        <v>121</v>
+      </c>
+      <c r="BX35"/>
+    </row>
+    <row r="36" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C36" s="17"/>
       <c r="D36" s="25" t="s">
         <v>5</v>
@@ -5733,8 +6060,19 @@
         <v>122</v>
       </c>
       <c r="BR36"/>
-    </row>
-    <row r="37" spans="3:70" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="BT36" s="51"/>
+      <c r="BU36">
+        <v>1</v>
+      </c>
+      <c r="BV36" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW36" t="s">
+        <v>122</v>
+      </c>
+      <c r="BX36"/>
+    </row>
+    <row r="37" spans="3:76" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C37" s="34"/>
       <c r="D37" s="35" t="s">
         <v>6</v>
@@ -5864,8 +6202,19 @@
         <v>123</v>
       </c>
       <c r="BR37"/>
-    </row>
-    <row r="38" spans="3:70" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="BT37" s="51"/>
+      <c r="BU37">
+        <v>1</v>
+      </c>
+      <c r="BV37" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW37" t="s">
+        <v>123</v>
+      </c>
+      <c r="BX37"/>
+    </row>
+    <row r="38" spans="3:76" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C38" s="17"/>
       <c r="D38"/>
       <c r="E38"/>
@@ -5927,8 +6276,13 @@
       <c r="BP38"/>
       <c r="BQ38"/>
       <c r="BR38"/>
-    </row>
-    <row r="39" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT38" s="51"/>
+      <c r="BU38"/>
+      <c r="BV38"/>
+      <c r="BW38"/>
+      <c r="BX38"/>
+    </row>
+    <row r="39" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C39" s="36" t="s">
         <v>24</v>
       </c>
@@ -5992,8 +6346,13 @@
       <c r="BP39"/>
       <c r="BQ39"/>
       <c r="BR39"/>
-    </row>
-    <row r="40" spans="3:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT39" s="51"/>
+      <c r="BU39"/>
+      <c r="BV39"/>
+      <c r="BW39"/>
+      <c r="BX39"/>
+    </row>
+    <row r="40" spans="3:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C40" s="27" t="s">
         <v>25</v>
       </c>
@@ -6080,8 +6439,15 @@
       <c r="BP40" s="29"/>
       <c r="BQ40" s="29"/>
       <c r="BR40" s="29"/>
-    </row>
-    <row r="41" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT40" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="BU40" s="29"/>
+      <c r="BV40" s="29"/>
+      <c r="BW40" s="29"/>
+      <c r="BX40" s="29"/>
+    </row>
+    <row r="41" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C41" s="17"/>
       <c r="D41" s="25" t="s">
         <v>3</v>
@@ -6211,8 +6577,19 @@
         <v>27</v>
       </c>
       <c r="BR41"/>
-    </row>
-    <row r="42" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT41" s="51"/>
+      <c r="BU41">
+        <v>1</v>
+      </c>
+      <c r="BV41" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW41" t="s">
+        <v>27</v>
+      </c>
+      <c r="BX41"/>
+    </row>
+    <row r="42" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C42" s="17"/>
       <c r="D42" s="25" t="s">
         <v>4</v>
@@ -6342,8 +6719,19 @@
         <v>28</v>
       </c>
       <c r="BR42"/>
-    </row>
-    <row r="43" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT42" s="51"/>
+      <c r="BU42">
+        <v>1</v>
+      </c>
+      <c r="BV42" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW42" t="s">
+        <v>28</v>
+      </c>
+      <c r="BX42"/>
+    </row>
+    <row r="43" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C43" s="17"/>
       <c r="D43" s="25" t="s">
         <v>5</v>
@@ -6473,8 +6861,19 @@
         <v>29</v>
       </c>
       <c r="BR43"/>
-    </row>
-    <row r="44" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT43" s="51"/>
+      <c r="BU43">
+        <v>1</v>
+      </c>
+      <c r="BV43" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW43" t="s">
+        <v>29</v>
+      </c>
+      <c r="BX43"/>
+    </row>
+    <row r="44" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C44" s="17"/>
       <c r="D44" s="25" t="s">
         <v>6</v>
@@ -6604,8 +7003,19 @@
         <v>30</v>
       </c>
       <c r="BR44"/>
-    </row>
-    <row r="45" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT44" s="51"/>
+      <c r="BU44">
+        <v>1</v>
+      </c>
+      <c r="BV44" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW44" t="s">
+        <v>30</v>
+      </c>
+      <c r="BX44"/>
+    </row>
+    <row r="45" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C45" s="17"/>
       <c r="D45" s="25" t="s">
         <v>13</v>
@@ -6669,8 +7079,13 @@
       <c r="BP45"/>
       <c r="BQ45"/>
       <c r="BR45"/>
-    </row>
-    <row r="46" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT45" s="51"/>
+      <c r="BU45"/>
+      <c r="BV45"/>
+      <c r="BW45"/>
+      <c r="BX45"/>
+    </row>
+    <row r="46" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C46" s="27" t="s">
         <v>256</v>
       </c>
@@ -6734,8 +7149,13 @@
       <c r="BP46"/>
       <c r="BQ46"/>
       <c r="BR46"/>
-    </row>
-    <row r="47" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT46" s="51"/>
+      <c r="BU46"/>
+      <c r="BV46"/>
+      <c r="BW46"/>
+      <c r="BX46"/>
+    </row>
+    <row r="47" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C47" s="17"/>
       <c r="D47" s="25" t="s">
         <v>3</v>
@@ -6799,8 +7219,13 @@
       <c r="BP47"/>
       <c r="BQ47"/>
       <c r="BR47"/>
-    </row>
-    <row r="48" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT47" s="51"/>
+      <c r="BU47"/>
+      <c r="BV47"/>
+      <c r="BW47"/>
+      <c r="BX47"/>
+    </row>
+    <row r="48" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C48" s="17"/>
       <c r="D48" s="25" t="s">
         <v>4</v>
@@ -6864,8 +7289,13 @@
       <c r="BP48"/>
       <c r="BQ48"/>
       <c r="BR48"/>
-    </row>
-    <row r="49" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT48" s="51"/>
+      <c r="BU48"/>
+      <c r="BV48"/>
+      <c r="BW48"/>
+      <c r="BX48"/>
+    </row>
+    <row r="49" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C49" s="17"/>
       <c r="D49" s="25" t="s">
         <v>5</v>
@@ -6929,8 +7359,13 @@
       <c r="BP49"/>
       <c r="BQ49"/>
       <c r="BR49"/>
-    </row>
-    <row r="50" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT49" s="51"/>
+      <c r="BU49"/>
+      <c r="BV49"/>
+      <c r="BW49"/>
+      <c r="BX49"/>
+    </row>
+    <row r="50" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C50" s="17"/>
       <c r="D50" s="25" t="s">
         <v>6</v>
@@ -7104,8 +7539,23 @@
       <c r="BR50" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="51" spans="2:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT50" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="BU50">
+        <v>1</v>
+      </c>
+      <c r="BV50" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW50" t="s">
+        <v>257</v>
+      </c>
+      <c r="BX50" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="51" spans="2:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C51" s="27" t="s">
         <v>31</v>
       </c>
@@ -7170,8 +7620,13 @@
       <c r="BP51" s="29"/>
       <c r="BQ51" s="29"/>
       <c r="BR51" s="29"/>
-    </row>
-    <row r="52" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT51" s="52"/>
+      <c r="BU51" s="29"/>
+      <c r="BV51" s="29"/>
+      <c r="BW51" s="29"/>
+      <c r="BX51" s="29"/>
+    </row>
+    <row r="52" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C52" s="17"/>
       <c r="D52" s="25" t="s">
         <v>3</v>
@@ -7323,8 +7778,21 @@
         <v>32</v>
       </c>
       <c r="BR52"/>
-    </row>
-    <row r="53" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT52" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="BU52">
+        <v>1</v>
+      </c>
+      <c r="BV52" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW52" t="s">
+        <v>32</v>
+      </c>
+      <c r="BX52"/>
+    </row>
+    <row r="53" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C53" s="17"/>
       <c r="D53" s="25" t="s">
         <v>4</v>
@@ -7476,8 +7944,21 @@
         <v>33</v>
       </c>
       <c r="BR53"/>
-    </row>
-    <row r="54" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT53" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="BU53">
+        <v>1</v>
+      </c>
+      <c r="BV53" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW53" t="s">
+        <v>33</v>
+      </c>
+      <c r="BX53"/>
+    </row>
+    <row r="54" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C54" s="17"/>
       <c r="D54" s="25" t="s">
         <v>5</v>
@@ -7629,8 +8110,21 @@
         <v>34</v>
       </c>
       <c r="BR54"/>
-    </row>
-    <row r="55" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT54" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="BU54">
+        <v>1</v>
+      </c>
+      <c r="BV54" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW54" t="s">
+        <v>34</v>
+      </c>
+      <c r="BX54"/>
+    </row>
+    <row r="55" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C55" s="17"/>
       <c r="D55" s="25" t="s">
         <v>6</v>
@@ -7782,8 +8276,21 @@
         <v>35</v>
       </c>
       <c r="BR55"/>
-    </row>
-    <row r="56" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT55" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="BU55">
+        <v>1</v>
+      </c>
+      <c r="BV55" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW55" t="s">
+        <v>35</v>
+      </c>
+      <c r="BX55"/>
+    </row>
+    <row r="56" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C56" s="17"/>
       <c r="D56" s="25" t="s">
         <v>13</v>
@@ -7847,8 +8354,13 @@
       <c r="BP56"/>
       <c r="BQ56"/>
       <c r="BR56"/>
-    </row>
-    <row r="57" spans="2:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT56" s="51"/>
+      <c r="BU56"/>
+      <c r="BV56"/>
+      <c r="BW56"/>
+      <c r="BX56"/>
+    </row>
+    <row r="57" spans="2:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C57" s="27" t="s">
         <v>36</v>
       </c>
@@ -7913,8 +8425,13 @@
       <c r="BP57" s="29"/>
       <c r="BQ57" s="29"/>
       <c r="BR57" s="29"/>
-    </row>
-    <row r="58" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT57" s="52"/>
+      <c r="BU57" s="29"/>
+      <c r="BV57" s="29"/>
+      <c r="BW57" s="29"/>
+      <c r="BX57" s="29"/>
+    </row>
+    <row r="58" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C58" s="17"/>
       <c r="D58" s="40" t="s">
         <v>3</v>
@@ -8044,8 +8561,19 @@
         <v>37</v>
       </c>
       <c r="BR58"/>
-    </row>
-    <row r="59" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT58" s="51"/>
+      <c r="BU58">
+        <v>2</v>
+      </c>
+      <c r="BV58" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW58" t="s">
+        <v>37</v>
+      </c>
+      <c r="BX58"/>
+    </row>
+    <row r="59" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C59" s="17"/>
       <c r="D59" s="40" t="s">
         <v>4</v>
@@ -8175,8 +8703,19 @@
         <v>38</v>
       </c>
       <c r="BR59"/>
-    </row>
-    <row r="60" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT59" s="51"/>
+      <c r="BU59">
+        <v>2</v>
+      </c>
+      <c r="BV59" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW59" t="s">
+        <v>38</v>
+      </c>
+      <c r="BX59"/>
+    </row>
+    <row r="60" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C60" s="17"/>
       <c r="D60" s="40" t="s">
         <v>5</v>
@@ -8306,8 +8845,19 @@
         <v>39</v>
       </c>
       <c r="BR60"/>
-    </row>
-    <row r="61" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT60" s="51"/>
+      <c r="BU60">
+        <v>2</v>
+      </c>
+      <c r="BV60" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW60" t="s">
+        <v>39</v>
+      </c>
+      <c r="BX60"/>
+    </row>
+    <row r="61" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C61" s="17"/>
       <c r="D61" s="40" t="s">
         <v>6</v>
@@ -8437,8 +8987,19 @@
         <v>40</v>
       </c>
       <c r="BR61"/>
-    </row>
-    <row r="62" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT61" s="51"/>
+      <c r="BU61">
+        <v>2</v>
+      </c>
+      <c r="BV61" t="s">
+        <v>131</v>
+      </c>
+      <c r="BW61" t="s">
+        <v>40</v>
+      </c>
+      <c r="BX61"/>
+    </row>
+    <row r="62" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C62" s="17"/>
       <c r="D62" s="40" t="s">
         <v>13</v>
@@ -8502,8 +9063,13 @@
       <c r="BP62"/>
       <c r="BQ62"/>
       <c r="BR62"/>
-    </row>
-    <row r="63" spans="2:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT62" s="51"/>
+      <c r="BU62"/>
+      <c r="BV62"/>
+      <c r="BW62"/>
+      <c r="BX62"/>
+    </row>
+    <row r="63" spans="2:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B63" s="6">
         <v>1</v>
       </c>
@@ -8571,8 +9137,13 @@
       <c r="BP63"/>
       <c r="BQ63" s="29"/>
       <c r="BR63" s="29"/>
-    </row>
-    <row r="64" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT63" s="52"/>
+      <c r="BU63"/>
+      <c r="BV63"/>
+      <c r="BW63" s="29"/>
+      <c r="BX63" s="29"/>
+    </row>
+    <row r="64" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C64" s="17"/>
       <c r="D64" s="40" t="s">
         <v>3</v>
@@ -8724,8 +9295,21 @@
         <v>290</v>
       </c>
       <c r="BR64"/>
-    </row>
-    <row r="65" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT64" s="53" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU64">
+        <v>1</v>
+      </c>
+      <c r="BV64" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW64" t="s">
+        <v>290</v>
+      </c>
+      <c r="BX64"/>
+    </row>
+    <row r="65" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C65" s="17"/>
       <c r="D65" s="40" t="s">
         <v>4</v>
@@ -8877,8 +9461,21 @@
         <v>291</v>
       </c>
       <c r="BR65"/>
-    </row>
-    <row r="66" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT65" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU65">
+        <v>1</v>
+      </c>
+      <c r="BV65" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW65" t="s">
+        <v>291</v>
+      </c>
+      <c r="BX65"/>
+    </row>
+    <row r="66" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C66" s="17"/>
       <c r="D66" s="40" t="s">
         <v>5</v>
@@ -9030,8 +9627,21 @@
         <v>292</v>
       </c>
       <c r="BR66"/>
-    </row>
-    <row r="67" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT66" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU66">
+        <v>1</v>
+      </c>
+      <c r="BV66" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW66" t="s">
+        <v>292</v>
+      </c>
+      <c r="BX66"/>
+    </row>
+    <row r="67" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C67" s="17"/>
       <c r="D67" s="40" t="s">
         <v>6</v>
@@ -9183,8 +9793,21 @@
         <v>293</v>
       </c>
       <c r="BR67"/>
-    </row>
-    <row r="68" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT67" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU67">
+        <v>1</v>
+      </c>
+      <c r="BV67" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW67" t="s">
+        <v>293</v>
+      </c>
+      <c r="BX67"/>
+    </row>
+    <row r="68" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C68" s="17"/>
       <c r="D68" s="40" t="s">
         <v>287</v>
@@ -9336,8 +9959,21 @@
         <v>288</v>
       </c>
       <c r="BR68"/>
-    </row>
-    <row r="69" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT68" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU68">
+        <v>1</v>
+      </c>
+      <c r="BV68" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW68" t="s">
+        <v>288</v>
+      </c>
+      <c r="BX68"/>
+    </row>
+    <row r="69" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C69" s="27" t="s">
         <v>132</v>
       </c>
@@ -9401,8 +10037,13 @@
       <c r="BP69" s="29"/>
       <c r="BQ69" s="29"/>
       <c r="BR69"/>
-    </row>
-    <row r="70" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT69" s="52"/>
+      <c r="BU69" s="29"/>
+      <c r="BV69" s="29"/>
+      <c r="BW69" s="29"/>
+      <c r="BX69"/>
+    </row>
+    <row r="70" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C70" s="17"/>
       <c r="D70" s="40" t="s">
         <v>3</v>
@@ -9554,8 +10195,21 @@
         <v>41</v>
       </c>
       <c r="BR70"/>
-    </row>
-    <row r="71" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT70" s="53" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU70">
+        <v>1</v>
+      </c>
+      <c r="BV70" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW70" t="s">
+        <v>41</v>
+      </c>
+      <c r="BX70"/>
+    </row>
+    <row r="71" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C71" s="17"/>
       <c r="D71" s="40" t="s">
         <v>4</v>
@@ -9707,8 +10361,21 @@
         <v>42</v>
       </c>
       <c r="BR71"/>
-    </row>
-    <row r="72" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT71" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU71">
+        <v>1</v>
+      </c>
+      <c r="BV71" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW71" t="s">
+        <v>42</v>
+      </c>
+      <c r="BX71"/>
+    </row>
+    <row r="72" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C72" s="17"/>
       <c r="D72" s="40" t="s">
         <v>5</v>
@@ -9860,8 +10527,21 @@
         <v>43</v>
       </c>
       <c r="BR72"/>
-    </row>
-    <row r="73" spans="3:70" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="BT72" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU72">
+        <v>1</v>
+      </c>
+      <c r="BV72" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW72" t="s">
+        <v>43</v>
+      </c>
+      <c r="BX72"/>
+    </row>
+    <row r="73" spans="3:76" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C73" s="17"/>
       <c r="D73" s="40" t="s">
         <v>6</v>
@@ -10013,8 +10693,21 @@
         <v>44</v>
       </c>
       <c r="BR73"/>
-    </row>
-    <row r="74" spans="3:70" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="BT73" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU73">
+        <v>1</v>
+      </c>
+      <c r="BV73" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW73" t="s">
+        <v>44</v>
+      </c>
+      <c r="BX73"/>
+    </row>
+    <row r="74" spans="3:76" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C74" s="17"/>
       <c r="D74" s="40" t="s">
         <v>287</v>
@@ -10166,8 +10859,21 @@
         <v>294</v>
       </c>
       <c r="BR74"/>
-    </row>
-    <row r="75" spans="3:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT74" s="54" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU74">
+        <v>1</v>
+      </c>
+      <c r="BV74" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW74" t="s">
+        <v>294</v>
+      </c>
+      <c r="BX74"/>
+    </row>
+    <row r="75" spans="3:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C75" s="27" t="s">
         <v>45</v>
       </c>
@@ -10232,8 +10938,13 @@
       <c r="BP75" s="29"/>
       <c r="BQ75" s="29"/>
       <c r="BR75" s="29"/>
-    </row>
-    <row r="76" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT75" s="52"/>
+      <c r="BU75" s="29"/>
+      <c r="BV75" s="29"/>
+      <c r="BW75" s="29"/>
+      <c r="BX75" s="29"/>
+    </row>
+    <row r="76" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C76" s="17"/>
       <c r="D76" s="40" t="s">
         <v>3</v>
@@ -10385,8 +11096,21 @@
         <v>133</v>
       </c>
       <c r="BR76"/>
-    </row>
-    <row r="77" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT76" s="52" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU76">
+        <v>1</v>
+      </c>
+      <c r="BV76" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW76" t="s">
+        <v>133</v>
+      </c>
+      <c r="BX76"/>
+    </row>
+    <row r="77" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C77" s="17"/>
       <c r="D77" s="40" t="s">
         <v>4</v>
@@ -10538,8 +11262,21 @@
         <v>134</v>
       </c>
       <c r="BR77"/>
-    </row>
-    <row r="78" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT77" s="52" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU77">
+        <v>1</v>
+      </c>
+      <c r="BV77" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW77" t="s">
+        <v>134</v>
+      </c>
+      <c r="BX77"/>
+    </row>
+    <row r="78" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C78" s="17"/>
       <c r="D78" s="40" t="s">
         <v>5</v>
@@ -10691,8 +11428,21 @@
         <v>135</v>
       </c>
       <c r="BR78"/>
-    </row>
-    <row r="79" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT78" s="52" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU78">
+        <v>1</v>
+      </c>
+      <c r="BV78" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW78" t="s">
+        <v>135</v>
+      </c>
+      <c r="BX78"/>
+    </row>
+    <row r="79" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C79" s="17"/>
       <c r="D79" s="40" t="s">
         <v>6</v>
@@ -10844,8 +11594,21 @@
         <v>136</v>
       </c>
       <c r="BR79"/>
-    </row>
-    <row r="80" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT79" s="52" t="s">
+        <v>127</v>
+      </c>
+      <c r="BU79">
+        <v>1</v>
+      </c>
+      <c r="BV79" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW79" t="s">
+        <v>136</v>
+      </c>
+      <c r="BX79"/>
+    </row>
+    <row r="80" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C80" s="17"/>
       <c r="D80" s="40" t="s">
         <v>13</v>
@@ -10909,8 +11672,13 @@
       <c r="BP80"/>
       <c r="BQ80"/>
       <c r="BR80"/>
-    </row>
-    <row r="81" spans="2:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT80" s="51"/>
+      <c r="BU80"/>
+      <c r="BV80"/>
+      <c r="BW80"/>
+      <c r="BX80"/>
+    </row>
+    <row r="81" spans="2:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C81" s="27" t="s">
         <v>46</v>
       </c>
@@ -10975,8 +11743,13 @@
       <c r="BP81" s="29"/>
       <c r="BQ81" s="29"/>
       <c r="BR81" s="29"/>
-    </row>
-    <row r="82" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT81" s="52"/>
+      <c r="BU81" s="29"/>
+      <c r="BV81" s="29"/>
+      <c r="BW81" s="29"/>
+      <c r="BX81" s="29"/>
+    </row>
+    <row r="82" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C82" s="17"/>
       <c r="D82" s="40" t="s">
         <v>3</v>
@@ -11128,8 +11901,21 @@
         <v>47</v>
       </c>
       <c r="BR82"/>
-    </row>
-    <row r="83" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT82" s="51" t="s">
+        <v>125</v>
+      </c>
+      <c r="BU82">
+        <v>0</v>
+      </c>
+      <c r="BV82" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW82" t="s">
+        <v>47</v>
+      </c>
+      <c r="BX82"/>
+    </row>
+    <row r="83" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C83" s="17"/>
       <c r="D83" s="40" t="s">
         <v>4</v>
@@ -11281,8 +12067,21 @@
         <v>48</v>
       </c>
       <c r="BR83" s="13"/>
-    </row>
-    <row r="84" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT83" s="51" t="s">
+        <v>125</v>
+      </c>
+      <c r="BU83">
+        <v>0</v>
+      </c>
+      <c r="BV83" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW83" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="BX83" s="13"/>
+    </row>
+    <row r="84" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C84" s="17"/>
       <c r="D84" s="40" t="s">
         <v>5</v>
@@ -11434,8 +12233,21 @@
         <v>49</v>
       </c>
       <c r="BR84" s="13"/>
-    </row>
-    <row r="85" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT84" s="51" t="s">
+        <v>125</v>
+      </c>
+      <c r="BU84">
+        <v>0</v>
+      </c>
+      <c r="BV84" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW84" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="BX84" s="13"/>
+    </row>
+    <row r="85" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C85" s="17"/>
       <c r="D85" s="40" t="s">
         <v>6</v>
@@ -11587,8 +12399,21 @@
         <v>50</v>
       </c>
       <c r="BR85" s="13"/>
-    </row>
-    <row r="86" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT85" s="51" t="s">
+        <v>125</v>
+      </c>
+      <c r="BU85">
+        <v>0</v>
+      </c>
+      <c r="BV85" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW85" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="BX85" s="13"/>
+    </row>
+    <row r="86" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C86" s="17"/>
       <c r="D86" s="40" t="s">
         <v>287</v>
@@ -11740,8 +12565,21 @@
         <v>51</v>
       </c>
       <c r="BR86" s="13"/>
-    </row>
-    <row r="87" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT86" s="51" t="s">
+        <v>125</v>
+      </c>
+      <c r="BU86">
+        <v>0</v>
+      </c>
+      <c r="BV86" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW86" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="BX86" s="13"/>
+    </row>
+    <row r="87" spans="2:76" x14ac:dyDescent="0.2">
       <c r="B87">
         <v>2</v>
       </c>
@@ -11808,8 +12646,13 @@
       <c r="BP87" s="29"/>
       <c r="BQ87" s="43"/>
       <c r="BR87" s="13"/>
-    </row>
-    <row r="88" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT87" s="52"/>
+      <c r="BU87" s="29"/>
+      <c r="BV87" s="29"/>
+      <c r="BW87" s="43"/>
+      <c r="BX87" s="13"/>
+    </row>
+    <row r="88" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C88" s="17"/>
       <c r="D88" s="40" t="s">
         <v>3</v>
@@ -11961,8 +12804,21 @@
         <v>47</v>
       </c>
       <c r="BR88"/>
-    </row>
-    <row r="89" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT88" s="51" t="s">
+        <v>124</v>
+      </c>
+      <c r="BU88">
+        <v>1</v>
+      </c>
+      <c r="BV88" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW88" t="s">
+        <v>47</v>
+      </c>
+      <c r="BX88"/>
+    </row>
+    <row r="89" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C89" s="17"/>
       <c r="D89" s="40" t="s">
         <v>4</v>
@@ -12114,8 +12970,21 @@
         <v>48</v>
       </c>
       <c r="BR89" s="13"/>
-    </row>
-    <row r="90" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT89" s="51" t="s">
+        <v>124</v>
+      </c>
+      <c r="BU89">
+        <v>1</v>
+      </c>
+      <c r="BV89" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW89" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="BX89" s="13"/>
+    </row>
+    <row r="90" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C90" s="17"/>
       <c r="D90" s="40" t="s">
         <v>5</v>
@@ -12267,8 +13136,21 @@
         <v>49</v>
       </c>
       <c r="BR90" s="13"/>
-    </row>
-    <row r="91" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT90" s="51" t="s">
+        <v>124</v>
+      </c>
+      <c r="BU90">
+        <v>1</v>
+      </c>
+      <c r="BV90" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW90" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="BX90" s="13"/>
+    </row>
+    <row r="91" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C91" s="17"/>
       <c r="D91" s="40" t="s">
         <v>6</v>
@@ -12420,8 +13302,21 @@
         <v>50</v>
       </c>
       <c r="BR91" s="13"/>
-    </row>
-    <row r="92" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT91" s="51" t="s">
+        <v>124</v>
+      </c>
+      <c r="BU91">
+        <v>1</v>
+      </c>
+      <c r="BV91" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW91" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="BX91" s="13"/>
+    </row>
+    <row r="92" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C92" s="17"/>
       <c r="D92" s="40" t="s">
         <v>287</v>
@@ -12573,8 +13468,21 @@
         <v>51</v>
       </c>
       <c r="BR92" s="13"/>
-    </row>
-    <row r="93" spans="2:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT92" s="51" t="s">
+        <v>124</v>
+      </c>
+      <c r="BU92">
+        <v>1</v>
+      </c>
+      <c r="BV92" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW92" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="BX92" s="13"/>
+    </row>
+    <row r="93" spans="2:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C93" s="27" t="s">
         <v>52</v>
       </c>
@@ -12639,8 +13547,13 @@
       <c r="BP93" s="29"/>
       <c r="BQ93" s="29"/>
       <c r="BR93" s="29"/>
-    </row>
-    <row r="94" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT93" s="52"/>
+      <c r="BU93" s="29"/>
+      <c r="BV93" s="29"/>
+      <c r="BW93" s="29"/>
+      <c r="BX93" s="29"/>
+    </row>
+    <row r="94" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C94" s="17"/>
       <c r="D94" s="40" t="s">
         <v>3</v>
@@ -12704,8 +13617,13 @@
       <c r="BP94"/>
       <c r="BQ94"/>
       <c r="BR94"/>
-    </row>
-    <row r="95" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT94" s="51"/>
+      <c r="BU94"/>
+      <c r="BV94"/>
+      <c r="BW94"/>
+      <c r="BX94"/>
+    </row>
+    <row r="95" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C95" s="17"/>
       <c r="D95" s="40" t="s">
         <v>4</v>
@@ -12769,8 +13687,13 @@
       <c r="BP95"/>
       <c r="BQ95"/>
       <c r="BR95"/>
-    </row>
-    <row r="96" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT95" s="51"/>
+      <c r="BU95"/>
+      <c r="BV95"/>
+      <c r="BW95"/>
+      <c r="BX95"/>
+    </row>
+    <row r="96" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C96" s="17"/>
       <c r="D96" s="40" t="s">
         <v>5</v>
@@ -12834,8 +13757,13 @@
       <c r="BP96"/>
       <c r="BQ96"/>
       <c r="BR96"/>
-    </row>
-    <row r="97" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT96" s="51"/>
+      <c r="BU96"/>
+      <c r="BV96"/>
+      <c r="BW96"/>
+      <c r="BX96"/>
+    </row>
+    <row r="97" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C97" s="17"/>
       <c r="D97" s="40" t="s">
         <v>6</v>
@@ -12965,8 +13893,19 @@
       <c r="BR97" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="98" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT97" s="51" t="s">
+        <v>124</v>
+      </c>
+      <c r="BU97"/>
+      <c r="BV97"/>
+      <c r="BW97" t="s">
+        <v>252</v>
+      </c>
+      <c r="BX97" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="98" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C98" s="17"/>
       <c r="D98" s="40" t="s">
         <v>13</v>
@@ -13030,8 +13969,13 @@
       <c r="BP98"/>
       <c r="BQ98"/>
       <c r="BR98"/>
-    </row>
-    <row r="99" spans="3:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT98" s="51"/>
+      <c r="BU98"/>
+      <c r="BV98"/>
+      <c r="BW98"/>
+      <c r="BX98"/>
+    </row>
+    <row r="99" spans="3:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C99" s="27" t="s">
         <v>53</v>
       </c>
@@ -13096,8 +14040,13 @@
       <c r="BP99" s="29"/>
       <c r="BQ99" s="29"/>
       <c r="BR99" s="29"/>
-    </row>
-    <row r="100" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT99" s="52"/>
+      <c r="BU99" s="29"/>
+      <c r="BV99" s="29"/>
+      <c r="BW99" s="29"/>
+      <c r="BX99" s="29"/>
+    </row>
+    <row r="100" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C100" s="17"/>
       <c r="D100" s="40" t="s">
         <v>3</v>
@@ -13205,8 +14154,17 @@
         <v>54</v>
       </c>
       <c r="BR100"/>
-    </row>
-    <row r="101" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT100" s="51"/>
+      <c r="BU100"/>
+      <c r="BV100" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW100" t="s">
+        <v>54</v>
+      </c>
+      <c r="BX100"/>
+    </row>
+    <row r="101" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C101" s="17"/>
       <c r="D101" s="40" t="s">
         <v>4</v>
@@ -13314,8 +14272,17 @@
         <v>55</v>
       </c>
       <c r="BR101"/>
-    </row>
-    <row r="102" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT101" s="51"/>
+      <c r="BU101"/>
+      <c r="BV101" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW101" t="s">
+        <v>55</v>
+      </c>
+      <c r="BX101"/>
+    </row>
+    <row r="102" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C102" s="17"/>
       <c r="D102" s="40" t="s">
         <v>5</v>
@@ -13423,8 +14390,17 @@
         <v>56</v>
       </c>
       <c r="BR102"/>
-    </row>
-    <row r="103" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT102" s="51"/>
+      <c r="BU102"/>
+      <c r="BV102" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW102" t="s">
+        <v>56</v>
+      </c>
+      <c r="BX102"/>
+    </row>
+    <row r="103" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C103" s="17"/>
       <c r="D103" s="40" t="s">
         <v>6</v>
@@ -13532,8 +14508,17 @@
         <v>57</v>
       </c>
       <c r="BR103"/>
-    </row>
-    <row r="104" spans="3:70" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="BT103" s="51"/>
+      <c r="BU103"/>
+      <c r="BV103" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW103" t="s">
+        <v>57</v>
+      </c>
+      <c r="BX103"/>
+    </row>
+    <row r="104" spans="3:76" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C104" s="34"/>
       <c r="D104" s="44" t="s">
         <v>13</v>
@@ -13597,8 +14582,13 @@
       <c r="BP104"/>
       <c r="BQ104"/>
       <c r="BR104"/>
-    </row>
-    <row r="105" spans="3:70" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="BT104" s="51"/>
+      <c r="BU104"/>
+      <c r="BV104"/>
+      <c r="BW104"/>
+      <c r="BX104"/>
+    </row>
+    <row r="105" spans="3:76" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C105" s="45"/>
       <c r="D105" s="46"/>
       <c r="E105" s="61"/>
@@ -13660,8 +14650,13 @@
       <c r="BP105"/>
       <c r="BQ105"/>
       <c r="BR105"/>
-    </row>
-    <row r="106" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT105" s="51"/>
+      <c r="BU105"/>
+      <c r="BV105"/>
+      <c r="BW105"/>
+      <c r="BX105"/>
+    </row>
+    <row r="106" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C106" s="36" t="s">
         <v>58</v>
       </c>
@@ -13725,8 +14720,13 @@
       <c r="BP106"/>
       <c r="BQ106"/>
       <c r="BR106"/>
-    </row>
-    <row r="107" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT106" s="51"/>
+      <c r="BU106"/>
+      <c r="BV106"/>
+      <c r="BW106"/>
+      <c r="BX106"/>
+    </row>
+    <row r="107" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C107" s="27"/>
       <c r="D107" s="48" t="s">
         <v>118</v>
@@ -13790,8 +14790,13 @@
       <c r="BP107"/>
       <c r="BQ107"/>
       <c r="BR107"/>
-    </row>
-    <row r="108" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT107" s="51"/>
+      <c r="BU107"/>
+      <c r="BV107"/>
+      <c r="BW107"/>
+      <c r="BX107"/>
+    </row>
+    <row r="108" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C108" s="27"/>
       <c r="D108" s="40" t="s">
         <v>3</v>
@@ -13921,8 +14926,19 @@
         <v>114</v>
       </c>
       <c r="BR108"/>
-    </row>
-    <row r="109" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT108" s="51"/>
+      <c r="BU108">
+        <v>2</v>
+      </c>
+      <c r="BV108" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW108" t="s">
+        <v>114</v>
+      </c>
+      <c r="BX108"/>
+    </row>
+    <row r="109" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C109" s="27"/>
       <c r="D109" s="40" t="s">
         <v>4</v>
@@ -14052,8 +15068,19 @@
         <v>117</v>
       </c>
       <c r="BR109"/>
-    </row>
-    <row r="110" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT109" s="51"/>
+      <c r="BU109">
+        <v>2</v>
+      </c>
+      <c r="BV109" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW109" t="s">
+        <v>117</v>
+      </c>
+      <c r="BX109"/>
+    </row>
+    <row r="110" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C110" s="27"/>
       <c r="D110" s="40" t="s">
         <v>5</v>
@@ -14183,8 +15210,19 @@
         <v>116</v>
       </c>
       <c r="BR110"/>
-    </row>
-    <row r="111" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT110" s="51"/>
+      <c r="BU110">
+        <v>2</v>
+      </c>
+      <c r="BV110" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW110" t="s">
+        <v>116</v>
+      </c>
+      <c r="BX110"/>
+    </row>
+    <row r="111" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C111" s="27"/>
       <c r="D111" s="40" t="s">
         <v>6</v>
@@ -14314,8 +15352,19 @@
         <v>115</v>
       </c>
       <c r="BR111"/>
-    </row>
-    <row r="112" spans="3:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT111" s="51"/>
+      <c r="BU111">
+        <v>2</v>
+      </c>
+      <c r="BV111" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW111" t="s">
+        <v>115</v>
+      </c>
+      <c r="BX111"/>
+    </row>
+    <row r="112" spans="3:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C112" s="27" t="s">
         <v>59</v>
       </c>
@@ -14380,8 +15429,13 @@
       <c r="BP112" s="29"/>
       <c r="BQ112" s="29"/>
       <c r="BR112" s="29"/>
-    </row>
-    <row r="113" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT112" s="52"/>
+      <c r="BU112" s="29"/>
+      <c r="BV112" s="29"/>
+      <c r="BW112" s="29"/>
+      <c r="BX112" s="29"/>
+    </row>
+    <row r="113" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C113" s="17"/>
       <c r="D113" s="40" t="s">
         <v>3</v>
@@ -14511,8 +15565,19 @@
         <v>60</v>
       </c>
       <c r="BR113"/>
-    </row>
-    <row r="114" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT113" s="51"/>
+      <c r="BU113">
+        <v>1</v>
+      </c>
+      <c r="BV113" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW113" t="s">
+        <v>60</v>
+      </c>
+      <c r="BX113"/>
+    </row>
+    <row r="114" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C114" s="17"/>
       <c r="D114" s="40" t="s">
         <v>4</v>
@@ -14642,8 +15707,19 @@
         <v>61</v>
       </c>
       <c r="BR114"/>
-    </row>
-    <row r="115" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT114" s="51"/>
+      <c r="BU114">
+        <v>1</v>
+      </c>
+      <c r="BV114" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW114" t="s">
+        <v>61</v>
+      </c>
+      <c r="BX114"/>
+    </row>
+    <row r="115" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C115" s="17"/>
       <c r="D115" s="40" t="s">
         <v>5</v>
@@ -14773,8 +15849,19 @@
         <v>62</v>
       </c>
       <c r="BR115"/>
-    </row>
-    <row r="116" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT115" s="51"/>
+      <c r="BU115">
+        <v>1</v>
+      </c>
+      <c r="BV115" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW115" t="s">
+        <v>62</v>
+      </c>
+      <c r="BX115"/>
+    </row>
+    <row r="116" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C116" s="17"/>
       <c r="D116" s="40" t="s">
         <v>6</v>
@@ -14904,8 +15991,19 @@
         <v>63</v>
       </c>
       <c r="BR116"/>
-    </row>
-    <row r="117" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT116" s="51"/>
+      <c r="BU116">
+        <v>1</v>
+      </c>
+      <c r="BV116" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW116" t="s">
+        <v>63</v>
+      </c>
+      <c r="BX116"/>
+    </row>
+    <row r="117" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C117" s="17"/>
       <c r="D117" s="40" t="s">
         <v>13</v>
@@ -15035,8 +16133,19 @@
         <v>64</v>
       </c>
       <c r="BR117"/>
-    </row>
-    <row r="118" spans="2:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT117" s="51"/>
+      <c r="BU117">
+        <v>1</v>
+      </c>
+      <c r="BV117" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW117" t="s">
+        <v>64</v>
+      </c>
+      <c r="BX117"/>
+    </row>
+    <row r="118" spans="2:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C118" s="27" t="s">
         <v>65</v>
       </c>
@@ -15101,8 +16210,13 @@
       <c r="BP118" s="29"/>
       <c r="BQ118" s="29"/>
       <c r="BR118" s="29"/>
-    </row>
-    <row r="119" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT118" s="52"/>
+      <c r="BU118" s="29"/>
+      <c r="BV118" s="29"/>
+      <c r="BW118" s="29"/>
+      <c r="BX118" s="29"/>
+    </row>
+    <row r="119" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C119" s="17"/>
       <c r="D119" s="40" t="s">
         <v>3</v>
@@ -15166,8 +16280,13 @@
       <c r="BP119"/>
       <c r="BQ119"/>
       <c r="BR119"/>
-    </row>
-    <row r="120" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT119" s="51"/>
+      <c r="BU119"/>
+      <c r="BV119"/>
+      <c r="BW119"/>
+      <c r="BX119"/>
+    </row>
+    <row r="120" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C120" s="17"/>
       <c r="D120" s="40" t="s">
         <v>4</v>
@@ -15231,8 +16350,13 @@
       <c r="BP120"/>
       <c r="BQ120"/>
       <c r="BR120"/>
-    </row>
-    <row r="121" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT120" s="51"/>
+      <c r="BU120"/>
+      <c r="BV120"/>
+      <c r="BW120"/>
+      <c r="BX120"/>
+    </row>
+    <row r="121" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C121" s="17"/>
       <c r="D121" s="40" t="s">
         <v>5</v>
@@ -15296,8 +16420,13 @@
       <c r="BP121"/>
       <c r="BQ121"/>
       <c r="BR121"/>
-    </row>
-    <row r="122" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT121" s="51"/>
+      <c r="BU121"/>
+      <c r="BV121"/>
+      <c r="BW121"/>
+      <c r="BX121"/>
+    </row>
+    <row r="122" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C122" s="17"/>
       <c r="D122" s="40" t="s">
         <v>6</v>
@@ -15405,8 +16534,17 @@
       <c r="BR122" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="123" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT122" s="51"/>
+      <c r="BU122"/>
+      <c r="BV122"/>
+      <c r="BW122" t="s">
+        <v>254</v>
+      </c>
+      <c r="BX122" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="123" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C123" s="17"/>
       <c r="D123" s="40" t="s">
         <v>13</v>
@@ -15470,8 +16608,13 @@
       <c r="BP123"/>
       <c r="BQ123"/>
       <c r="BR123"/>
-    </row>
-    <row r="124" spans="2:70" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT123" s="51"/>
+      <c r="BU123"/>
+      <c r="BV123"/>
+      <c r="BW123"/>
+      <c r="BX123"/>
+    </row>
+    <row r="124" spans="2:76" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B124" s="6">
         <v>3</v>
       </c>
@@ -15539,8 +16682,13 @@
       <c r="BP124" s="29"/>
       <c r="BQ124" s="29"/>
       <c r="BR124" s="29"/>
-    </row>
-    <row r="125" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT124" s="52"/>
+      <c r="BU124" s="29"/>
+      <c r="BV124" s="29"/>
+      <c r="BW124" s="29"/>
+      <c r="BX124" s="29"/>
+    </row>
+    <row r="125" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C125" s="17"/>
       <c r="D125" s="40" t="s">
         <v>3</v>
@@ -15692,8 +16840,21 @@
         <v>67</v>
       </c>
       <c r="BR125" s="13"/>
-    </row>
-    <row r="126" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT125" s="51" t="s">
+        <v>138</v>
+      </c>
+      <c r="BU125">
+        <v>1</v>
+      </c>
+      <c r="BV125" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW125" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="BX125" s="13"/>
+    </row>
+    <row r="126" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C126" s="17"/>
       <c r="D126" s="40" t="s">
         <v>4</v>
@@ -15823,8 +16984,19 @@
         <v>68</v>
       </c>
       <c r="BR126"/>
-    </row>
-    <row r="127" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT126" s="51"/>
+      <c r="BU126">
+        <v>1</v>
+      </c>
+      <c r="BV126" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW126" t="s">
+        <v>68</v>
+      </c>
+      <c r="BX126"/>
+    </row>
+    <row r="127" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C127" s="17"/>
       <c r="D127" s="40" t="s">
         <v>5</v>
@@ -15954,8 +17126,19 @@
         <v>69</v>
       </c>
       <c r="BR127"/>
-    </row>
-    <row r="128" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT127" s="51"/>
+      <c r="BU127">
+        <v>1</v>
+      </c>
+      <c r="BV127" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW127" t="s">
+        <v>69</v>
+      </c>
+      <c r="BX127"/>
+    </row>
+    <row r="128" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C128" s="27"/>
       <c r="D128" s="48" t="s">
         <v>6</v>
@@ -16107,8 +17290,21 @@
         <v>70</v>
       </c>
       <c r="BR128" s="13"/>
-    </row>
-    <row r="129" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT128" s="52" t="s">
+        <v>138</v>
+      </c>
+      <c r="BU128" s="29">
+        <v>1</v>
+      </c>
+      <c r="BV128" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW128" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="BX128" s="13"/>
+    </row>
+    <row r="129" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C129" s="9"/>
       <c r="D129" s="40" t="s">
         <v>287</v>
@@ -16224,8 +17420,18 @@
         <v>71</v>
       </c>
       <c r="BR129" s="13"/>
-    </row>
-    <row r="130" spans="2:70" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="BU129" s="1">
+        <v>1</v>
+      </c>
+      <c r="BV129" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW129" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="BX129" s="13"/>
+    </row>
+    <row r="130" spans="2:76" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C130" s="5" t="s">
         <v>72</v>
       </c>
@@ -16234,7 +17440,7 @@
       <c r="Q130" s="57"/>
       <c r="AC130" s="7"/>
     </row>
-    <row r="131" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C131" s="9"/>
       <c r="D131" s="11" t="s">
         <v>3</v>
@@ -16262,22 +17468,24 @@
       <c r="BJ131" s="13"/>
       <c r="BN131" s="51"/>
       <c r="BP131" s="13"/>
-    </row>
-    <row r="132" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT131" s="51"/>
+      <c r="BV131" s="13"/>
+    </row>
+    <row r="132" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C132" s="9"/>
       <c r="D132" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E132" s="62"/>
     </row>
-    <row r="133" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C133" s="9"/>
       <c r="D133" s="11" t="s">
         <v>5</v>
       </c>
       <c r="E133" s="62"/>
     </row>
-    <row r="134" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C134" s="9"/>
       <c r="D134" s="11" t="s">
         <v>6</v>
@@ -16442,15 +17650,30 @@
       <c r="BR134" s="1" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="135" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT134" s="51" t="s">
+        <v>138</v>
+      </c>
+      <c r="BU134" s="1">
+        <v>1</v>
+      </c>
+      <c r="BV134" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW134" t="s">
+        <v>255</v>
+      </c>
+      <c r="BX134" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="135" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C135" s="9"/>
       <c r="D135" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E135" s="62"/>
     </row>
-    <row r="136" spans="2:70" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:76" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="B136" s="6">
         <v>4</v>
       </c>
@@ -16462,7 +17685,7 @@
       <c r="Q136" s="57"/>
       <c r="AC136" s="7"/>
     </row>
-    <row r="137" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C137" s="9"/>
       <c r="D137" s="11" t="s">
         <v>3</v>
@@ -16567,8 +17790,17 @@
       <c r="BQ137" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="138" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BU137" s="1">
+        <v>1</v>
+      </c>
+      <c r="BV137" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW137" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="138" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C138" s="9"/>
       <c r="D138" s="11" t="s">
         <v>4</v>
@@ -16673,8 +17905,17 @@
       <c r="BQ138" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="139" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BU138" s="1">
+        <v>1</v>
+      </c>
+      <c r="BV138" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW138" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="139" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C139" s="9"/>
       <c r="D139" s="11" t="s">
         <v>5</v>
@@ -16779,8 +18020,17 @@
       <c r="BQ139" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="140" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BU139" s="1">
+        <v>1</v>
+      </c>
+      <c r="BV139" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW139" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="140" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C140" s="9"/>
       <c r="D140" s="11" t="s">
         <v>6</v>
@@ -16885,8 +18135,17 @@
       <c r="BQ140" s="1" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="141" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BU140" s="1">
+        <v>1</v>
+      </c>
+      <c r="BV140" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW140" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="141" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C141" s="9"/>
       <c r="D141" s="40" t="s">
         <v>287</v>
@@ -17002,8 +18261,18 @@
         <v>78</v>
       </c>
       <c r="BR141"/>
-    </row>
-    <row r="142" spans="2:70" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="BU141" s="1">
+        <v>1</v>
+      </c>
+      <c r="BV141" t="s">
+        <v>130</v>
+      </c>
+      <c r="BW141" t="s">
+        <v>78</v>
+      </c>
+      <c r="BX141"/>
+    </row>
+    <row r="142" spans="2:76" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C142" s="5" t="s">
         <v>79</v>
       </c>
@@ -17012,7 +18281,7 @@
       <c r="Q142" s="57"/>
       <c r="AC142" s="7"/>
     </row>
-    <row r="143" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C143" s="9"/>
       <c r="D143" s="11" t="s">
         <v>3</v>
@@ -17084,8 +18353,14 @@
       <c r="BQ143" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="144" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BV143" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW143" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="144" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C144" s="9"/>
       <c r="D144" s="11" t="s">
         <v>4</v>
@@ -17157,8 +18432,14 @@
       <c r="BQ144" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="145" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV144" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW144" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="145" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C145" s="9"/>
       <c r="D145" s="11" t="s">
         <v>5</v>
@@ -17230,8 +18511,14 @@
       <c r="BQ145" s="1" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="146" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV145" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW145" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="146" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C146" s="9"/>
       <c r="D146" s="11" t="s">
         <v>6</v>
@@ -17303,15 +18590,21 @@
       <c r="BQ146" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="147" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV146" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW146" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="147" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C147" s="9"/>
       <c r="D147" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E147" s="62"/>
     </row>
-    <row r="148" spans="3:70" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+    <row r="148" spans="3:76" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C148" s="5" t="s">
         <v>84</v>
       </c>
@@ -17320,49 +18613,49 @@
       <c r="Q148" s="57"/>
       <c r="AC148" s="7"/>
     </row>
-    <row r="149" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="149" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C149" s="9"/>
       <c r="D149" s="11" t="s">
         <v>3</v>
       </c>
       <c r="E149" s="62"/>
     </row>
-    <row r="150" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="150" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C150" s="9"/>
       <c r="D150" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E150" s="62"/>
     </row>
-    <row r="151" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="151" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C151" s="9"/>
       <c r="D151" s="11" t="s">
         <v>5</v>
       </c>
       <c r="E151" s="62"/>
     </row>
-    <row r="152" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="152" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C152" s="9"/>
       <c r="D152" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E152" s="62"/>
     </row>
-    <row r="153" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="153" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C153" s="9"/>
       <c r="D153" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E153" s="62"/>
     </row>
-    <row r="154" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="154" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C154" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D154" s="10"/>
       <c r="E154" s="63"/>
     </row>
-    <row r="155" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="155" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C155" s="9"/>
       <c r="D155" s="11" t="s">
         <v>3</v>
@@ -17445,8 +18738,15 @@
         <v>86</v>
       </c>
       <c r="BR155"/>
-    </row>
-    <row r="156" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV155" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW155" t="s">
+        <v>86</v>
+      </c>
+      <c r="BX155"/>
+    </row>
+    <row r="156" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C156" s="9"/>
       <c r="D156" s="11" t="s">
         <v>4</v>
@@ -17529,8 +18829,15 @@
         <v>87</v>
       </c>
       <c r="BR156"/>
-    </row>
-    <row r="157" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV156" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW156" t="s">
+        <v>87</v>
+      </c>
+      <c r="BX156"/>
+    </row>
+    <row r="157" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C157" s="9"/>
       <c r="D157" s="11" t="s">
         <v>5</v>
@@ -17613,8 +18920,15 @@
         <v>88</v>
       </c>
       <c r="BR157"/>
-    </row>
-    <row r="158" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV157" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW157" t="s">
+        <v>88</v>
+      </c>
+      <c r="BX157"/>
+    </row>
+    <row r="158" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C158" s="9"/>
       <c r="D158" s="11" t="s">
         <v>6</v>
@@ -17697,26 +19011,33 @@
         <v>89</v>
       </c>
       <c r="BR158"/>
-    </row>
-    <row r="159" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV158" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW158" t="s">
+        <v>89</v>
+      </c>
+      <c r="BX158"/>
+    </row>
+    <row r="159" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C159" s="9"/>
       <c r="D159" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E159" s="62"/>
     </row>
-    <row r="160" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="160" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D160" s="59"/>
       <c r="E160" s="59"/>
     </row>
-    <row r="161" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="161" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C161" s="5" t="s">
         <v>295</v>
       </c>
       <c r="D161" s="59"/>
       <c r="E161" s="59"/>
     </row>
-    <row r="162" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="162" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D162" s="11" t="s">
         <v>6</v>
       </c>
@@ -17853,16 +19174,28 @@
       <c r="BR162" s="1" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="163" spans="3:70" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BU162" s="1">
+        <v>1</v>
+      </c>
+      <c r="BV162" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW162" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="BX162" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="163" spans="3:76" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C164" s="4" t="s">
         <v>90</v>
       </c>
       <c r="D164" s="12"/>
       <c r="E164" s="62"/>
     </row>
-    <row r="165" spans="3:70" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+    <row r="165" spans="3:76" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C165" s="5" t="s">
         <v>59</v>
       </c>
@@ -17871,7 +19204,7 @@
       <c r="Q165" s="57"/>
       <c r="AC165" s="7"/>
     </row>
-    <row r="166" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="166" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C166" s="9"/>
       <c r="D166" s="11" t="s">
         <v>3</v>
@@ -17943,8 +19276,14 @@
       <c r="BQ166" s="1" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="167" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV166" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW166" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="167" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C167" s="9"/>
       <c r="D167" s="11" t="s">
         <v>4</v>
@@ -18016,8 +19355,14 @@
       <c r="BQ167" s="1" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="168" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV167" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW167" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="168" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C168" s="9"/>
       <c r="D168" s="11" t="s">
         <v>5</v>
@@ -18089,8 +19434,14 @@
       <c r="BQ168" s="1" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="169" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV168" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW168" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="169" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C169" s="9"/>
       <c r="D169" s="11" t="s">
         <v>6</v>
@@ -18162,8 +19513,14 @@
       <c r="BQ169" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="170" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV169" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW169" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="170" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C170" s="9"/>
       <c r="D170" s="11" t="s">
         <v>13</v>
@@ -18202,8 +19559,11 @@
       <c r="BQ170" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="171" spans="3:70" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="BW170" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="171" spans="3:76" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C171" s="5" t="s">
         <v>65</v>
       </c>
@@ -18212,28 +19572,28 @@
       <c r="Q171" s="57"/>
       <c r="AC171" s="7"/>
     </row>
-    <row r="172" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="172" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C172" s="9"/>
       <c r="D172" s="11" t="s">
         <v>3</v>
       </c>
       <c r="E172" s="62"/>
     </row>
-    <row r="173" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="173" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C173" s="9"/>
       <c r="D173" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E173" s="62"/>
     </row>
-    <row r="174" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="174" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C174" s="9"/>
       <c r="D174" s="11" t="s">
         <v>5</v>
       </c>
       <c r="E174" s="62"/>
     </row>
-    <row r="175" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="175" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C175" s="17"/>
       <c r="D175" s="40" t="s">
         <v>6</v>
@@ -18407,15 +19767,30 @@
       <c r="BR175" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="176" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BT175" s="51" t="s">
+        <v>249</v>
+      </c>
+      <c r="BU175">
+        <v>1</v>
+      </c>
+      <c r="BV175" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW175" t="s">
+        <v>258</v>
+      </c>
+      <c r="BX175" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="176" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C176" s="9"/>
       <c r="D176" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E176" s="62"/>
     </row>
-    <row r="177" spans="3:69" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+    <row r="177" spans="3:75" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C177" s="5" t="s">
         <v>66</v>
       </c>
@@ -18424,7 +19799,7 @@
       <c r="Q177" s="57"/>
       <c r="AC177" s="7"/>
     </row>
-    <row r="178" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="178" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C178" s="9"/>
       <c r="D178" s="11" t="s">
         <v>3</v>
@@ -18496,8 +19871,14 @@
       <c r="BQ178" s="1" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="179" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV178" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW178" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="179" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C179" s="9"/>
       <c r="D179" s="11" t="s">
         <v>4</v>
@@ -18569,8 +19950,14 @@
       <c r="BQ179" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="180" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV179" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW179" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="180" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C180" s="9"/>
       <c r="D180" s="11" t="s">
         <v>5</v>
@@ -18642,8 +20029,14 @@
       <c r="BQ180" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="181" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV180" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW180" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="181" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C181" s="9"/>
       <c r="D181" s="11" t="s">
         <v>6</v>
@@ -18715,15 +20108,21 @@
       <c r="BQ181" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="182" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV181" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW181" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="182" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C182" s="9"/>
       <c r="D182" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E182" s="62"/>
     </row>
-    <row r="183" spans="3:69" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+    <row r="183" spans="3:75" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C183" s="5" t="s">
         <v>72</v>
       </c>
@@ -18732,28 +20131,28 @@
       <c r="Q183" s="57"/>
       <c r="AC183" s="7"/>
     </row>
-    <row r="184" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="184" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C184" s="9"/>
       <c r="D184" s="11" t="s">
         <v>3</v>
       </c>
       <c r="E184" s="62"/>
     </row>
-    <row r="185" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="185" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C185" s="9"/>
       <c r="D185" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E185" s="62"/>
     </row>
-    <row r="186" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="186" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C186" s="9"/>
       <c r="D186" s="11" t="s">
         <v>5</v>
       </c>
       <c r="E186" s="62"/>
     </row>
-    <row r="187" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="187" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C187" s="9"/>
       <c r="D187" s="11" t="s">
         <v>6</v>
@@ -18873,15 +20272,24 @@
       <c r="BP187" s="13" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="188" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BT187" s="51" t="s">
+        <v>138</v>
+      </c>
+      <c r="BU187" s="1">
+        <v>1</v>
+      </c>
+      <c r="BV187" s="13" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="188" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C188" s="9"/>
       <c r="D188" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E188" s="62"/>
     </row>
-    <row r="189" spans="3:69" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+    <row r="189" spans="3:75" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C189" s="5" t="s">
         <v>73</v>
       </c>
@@ -18890,7 +20298,7 @@
       <c r="Q189" s="57"/>
       <c r="AC189" s="7"/>
     </row>
-    <row r="190" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="190" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C190" s="9"/>
       <c r="D190" s="11" t="s">
         <v>3</v>
@@ -18962,8 +20370,14 @@
       <c r="BQ190" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="191" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV190" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW190" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="191" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C191" s="9"/>
       <c r="D191" s="11" t="s">
         <v>4</v>
@@ -19035,8 +20449,14 @@
       <c r="BQ191" s="1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="192" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV191" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW191" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="192" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C192" s="9"/>
       <c r="D192" s="11" t="s">
         <v>5</v>
@@ -19108,8 +20528,14 @@
       <c r="BQ192" s="1" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="193" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV192" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW192" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="193" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C193" s="9"/>
       <c r="D193" s="11" t="s">
         <v>6</v>
@@ -19181,8 +20607,14 @@
       <c r="BQ193" s="1" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="194" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV193" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW193" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="194" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C194" s="9"/>
       <c r="D194" s="11" t="s">
         <v>13</v>
@@ -19254,8 +20686,14 @@
       <c r="BQ194" s="1" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="195" spans="3:69" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="BV194" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW194" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="195" spans="3:75" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C195" s="5" t="s">
         <v>79</v>
       </c>
@@ -19264,7 +20702,7 @@
       <c r="Q195" s="57"/>
       <c r="AC195" s="7"/>
     </row>
-    <row r="196" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="196" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C196" s="9"/>
       <c r="D196" s="11" t="s">
         <v>3</v>
@@ -19336,8 +20774,14 @@
       <c r="BQ196" s="1" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="197" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV196" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW196" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="197" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C197" s="9"/>
       <c r="D197" s="11" t="s">
         <v>4</v>
@@ -19409,8 +20853,14 @@
       <c r="BQ197" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="198" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV197" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW197" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="198" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C198" s="9"/>
       <c r="D198" s="11" t="s">
         <v>5</v>
@@ -19482,8 +20932,14 @@
       <c r="BQ198" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="199" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV198" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW198" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="199" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C199" s="9"/>
       <c r="D199" s="11" t="s">
         <v>6</v>
@@ -19555,8 +21011,14 @@
       <c r="BQ199" s="1" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="200" spans="3:69" x14ac:dyDescent="0.2">
+      <c r="BV199" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW199" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="200" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C200" s="9"/>
       <c r="D200" s="11" t="s">
         <v>13</v>
@@ -19628,8 +21090,14 @@
       <c r="BQ200" s="1" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="201" spans="3:69" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="BV200" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW200" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="201" spans="3:75" s="6" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C201" s="5" t="s">
         <v>84</v>
       </c>
@@ -19638,49 +21106,49 @@
       <c r="Q201" s="57"/>
       <c r="AC201" s="7"/>
     </row>
-    <row r="202" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="202" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C202" s="9"/>
       <c r="D202" s="11" t="s">
         <v>3</v>
       </c>
       <c r="E202" s="62"/>
     </row>
-    <row r="203" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="203" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C203" s="9"/>
       <c r="D203" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E203" s="62"/>
     </row>
-    <row r="204" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="204" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C204" s="9"/>
       <c r="D204" s="11" t="s">
         <v>5</v>
       </c>
       <c r="E204" s="62"/>
     </row>
-    <row r="205" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="205" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C205" s="9"/>
       <c r="D205" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E205" s="62"/>
     </row>
-    <row r="206" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="206" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C206" s="9"/>
       <c r="D206" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E206" s="62"/>
     </row>
-    <row r="207" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="207" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C207" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D207" s="10"/>
       <c r="E207" s="63"/>
     </row>
-    <row r="208" spans="3:69" x14ac:dyDescent="0.2">
+    <row r="208" spans="3:75" x14ac:dyDescent="0.2">
       <c r="C208" s="9"/>
       <c r="D208" s="11" t="s">
         <v>3</v>
@@ -19765,8 +21233,16 @@
       <c r="BQ208" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="209" spans="2:70" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BT208" s="2"/>
+      <c r="BU208" s="2"/>
+      <c r="BV208" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW208" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="209" spans="2:76" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B209"/>
       <c r="C209" s="9"/>
       <c r="D209" s="11" t="s">
@@ -19868,8 +21344,15 @@
         <v>110</v>
       </c>
       <c r="BR209"/>
-    </row>
-    <row r="210" spans="2:70" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BV209" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW209" t="s">
+        <v>110</v>
+      </c>
+      <c r="BX209"/>
+    </row>
+    <row r="210" spans="2:76" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B210"/>
       <c r="C210" s="9"/>
       <c r="D210" s="11" t="s">
@@ -19971,8 +21454,15 @@
         <v>111</v>
       </c>
       <c r="BR210"/>
-    </row>
-    <row r="211" spans="2:70" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BV210" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW210" t="s">
+        <v>111</v>
+      </c>
+      <c r="BX210"/>
+    </row>
+    <row r="211" spans="2:76" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B211"/>
       <c r="C211" s="9"/>
       <c r="D211" s="11" t="s">
@@ -20074,8 +21564,15 @@
         <v>112</v>
       </c>
       <c r="BR211"/>
-    </row>
-    <row r="212" spans="2:70" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="BV211" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW211" t="s">
+        <v>112</v>
+      </c>
+      <c r="BX211"/>
+    </row>
+    <row r="212" spans="2:76" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B212"/>
       <c r="C212" s="9"/>
       <c r="D212" s="11" t="s">
@@ -20136,13 +21633,18 @@
       <c r="BP212" s="1"/>
       <c r="BQ212" s="1"/>
       <c r="BR212"/>
-    </row>
-    <row r="213" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BT212" s="1"/>
+      <c r="BU212" s="1"/>
+      <c r="BV212" s="1"/>
+      <c r="BW212" s="1"/>
+      <c r="BX212"/>
+    </row>
+    <row r="213" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C213" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="214" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="214" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D214" s="11" t="s">
         <v>3</v>
       </c>
@@ -20230,8 +21732,12 @@
         <v>129</v>
       </c>
       <c r="BQ214"/>
-    </row>
-    <row r="215" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BV214" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW214"/>
+    </row>
+    <row r="215" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D215" s="11" t="s">
         <v>4</v>
       </c>
@@ -20320,8 +21826,13 @@
       </c>
       <c r="BQ215"/>
       <c r="BR215"/>
-    </row>
-    <row r="216" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BV215" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW215"/>
+      <c r="BX215"/>
+    </row>
+    <row r="216" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D216" s="11" t="s">
         <v>5</v>
       </c>
@@ -20410,8 +21921,13 @@
       </c>
       <c r="BQ216"/>
       <c r="BR216"/>
-    </row>
-    <row r="217" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BV216" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW216"/>
+      <c r="BX216"/>
+    </row>
+    <row r="217" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D217" s="11" t="s">
         <v>6</v>
       </c>
@@ -20500,22 +22016,28 @@
       </c>
       <c r="BQ217"/>
       <c r="BR217"/>
-    </row>
-    <row r="218" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BV217" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW217"/>
+      <c r="BX217"/>
+    </row>
+    <row r="218" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D218" s="11" t="s">
         <v>13</v>
       </c>
       <c r="E218" s="62"/>
       <c r="AY218" s="2"/>
       <c r="BR218"/>
-    </row>
-    <row r="219" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BX218"/>
+    </row>
+    <row r="219" spans="2:76" x14ac:dyDescent="0.2">
       <c r="C219" s="1" t="s">
         <v>181</v>
       </c>
       <c r="AY219" s="2"/>
     </row>
-    <row r="220" spans="2:70" x14ac:dyDescent="0.2">
+    <row r="220" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D220" s="11" t="s">
         <v>3</v>
       </c>
@@ -20596,8 +22118,14 @@
       <c r="BQ220" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="221" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BV220" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW220" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="221" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D221" s="11" t="s">
         <v>4</v>
       </c>
@@ -20679,8 +22207,15 @@
         <v>213</v>
       </c>
       <c r="BR221"/>
-    </row>
-    <row r="222" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BV221" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW221" t="s">
+        <v>213</v>
+      </c>
+      <c r="BX221"/>
+    </row>
+    <row r="222" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D222" s="11" t="s">
         <v>5</v>
       </c>
@@ -20762,8 +22297,15 @@
         <v>214</v>
       </c>
       <c r="BR222"/>
-    </row>
-    <row r="223" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BV222" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW222" t="s">
+        <v>214</v>
+      </c>
+      <c r="BX222"/>
+    </row>
+    <row r="223" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D223" s="11" t="s">
         <v>6</v>
       </c>
@@ -20845,8 +22387,15 @@
         <v>215</v>
       </c>
       <c r="BR223"/>
-    </row>
-    <row r="224" spans="2:70" x14ac:dyDescent="0.2">
+      <c r="BV223" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW223" t="s">
+        <v>215</v>
+      </c>
+      <c r="BX223"/>
+    </row>
+    <row r="224" spans="2:76" x14ac:dyDescent="0.2">
       <c r="D224" s="11" t="s">
         <v>13</v>
       </c>
@@ -20855,13 +22404,15 @@
       <c r="BL224"/>
       <c r="BQ224"/>
       <c r="BR224"/>
-    </row>
-    <row r="225" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BW224"/>
+      <c r="BX224"/>
+    </row>
+    <row r="225" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C225" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="226" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="226" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D226" s="11" t="s">
         <v>3</v>
       </c>
@@ -20885,7 +22436,7 @@
       <c r="BE226"/>
       <c r="BF226"/>
     </row>
-    <row r="227" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="227" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D227" s="11" t="s">
         <v>4</v>
       </c>
@@ -20912,8 +22463,10 @@
       <c r="BL227"/>
       <c r="BQ227"/>
       <c r="BR227"/>
-    </row>
-    <row r="228" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BW227"/>
+      <c r="BX227"/>
+    </row>
+    <row r="228" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D228" s="11" t="s">
         <v>5</v>
       </c>
@@ -20940,8 +22493,10 @@
       <c r="BL228"/>
       <c r="BQ228"/>
       <c r="BR228"/>
-    </row>
-    <row r="229" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BW228"/>
+      <c r="BX228"/>
+    </row>
+    <row r="229" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D229" s="11" t="s">
         <v>6</v>
       </c>
@@ -21041,8 +22596,13 @@
       </c>
       <c r="BQ229"/>
       <c r="BR229"/>
-    </row>
-    <row r="230" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV229" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW229"/>
+      <c r="BX229"/>
+    </row>
+    <row r="230" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D230" s="11" t="s">
         <v>13</v>
       </c>
@@ -21052,14 +22612,16 @@
       <c r="BL230"/>
       <c r="BQ230"/>
       <c r="BR230"/>
-    </row>
-    <row r="231" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BW230"/>
+      <c r="BX230"/>
+    </row>
+    <row r="231" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C231" s="1" t="s">
         <v>251</v>
       </c>
       <c r="AY231" s="2"/>
     </row>
-    <row r="232" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="232" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D232" s="11" t="s">
         <v>3</v>
       </c>
@@ -21085,8 +22647,9 @@
       <c r="BK232"/>
       <c r="BL232"/>
       <c r="BQ232"/>
-    </row>
-    <row r="233" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BW232"/>
+    </row>
+    <row r="233" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D233" s="11" t="s">
         <v>4</v>
       </c>
@@ -21113,8 +22676,10 @@
       <c r="BL233"/>
       <c r="BQ233"/>
       <c r="BR233"/>
-    </row>
-    <row r="234" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BW233"/>
+      <c r="BX233"/>
+    </row>
+    <row r="234" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D234" s="11" t="s">
         <v>5</v>
       </c>
@@ -21141,8 +22706,10 @@
       <c r="BL234"/>
       <c r="BQ234"/>
       <c r="BR234"/>
-    </row>
-    <row r="235" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BW234"/>
+      <c r="BX234"/>
+    </row>
+    <row r="235" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D235" s="11" t="s">
         <v>6</v>
       </c>
@@ -21248,8 +22815,17 @@
       <c r="BR235" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="236" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BV235" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BW235" t="s">
+        <v>264</v>
+      </c>
+      <c r="BX235" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="236" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D236" s="11" t="s">
         <v>13</v>
       </c>
@@ -21258,13 +22834,15 @@
       <c r="BL236"/>
       <c r="BQ236"/>
       <c r="BR236"/>
-    </row>
-    <row r="237" spans="3:70" x14ac:dyDescent="0.2">
+      <c r="BW236"/>
+      <c r="BX236"/>
+    </row>
+    <row r="237" spans="3:76" x14ac:dyDescent="0.2">
       <c r="C237" s="1" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="238" spans="3:70" x14ac:dyDescent="0.2">
+    <row r="238" spans="3:76" x14ac:dyDescent="0.2">
       <c r="D238" s="11" t="s">
         <v>6</v>
       </c>

</xml_diff>